<commit_message>
Add RQ3 design intervention (Study 2) + norming SOP/gold key for annotation
- methods_results_skeleton.docx: new Study 2 section — a Mechanism-Gap Report
  (correct conclusion + the specific flawed mechanism the defense exposed + quote
  + what-to-reteach) vs a plain mastery score, in a within-subject controlled
  study on the existing 106 episodes (no redeployment), testing whether it changes
  teachers' identification of hollow-but-MC-passing students and their
  instructional targeting; subject moderation ties RQ2<->RQ3. Lifts the validity
  audit into an artifact + empirical HCI contribution.
- gen_validity_packets.py: each packet now ships 编码手册 + 评分SOP + 对齐练习(8) +
  标注表; emits deliverables/norming_goldkey.md (facilitator) — 8 real norming
  episodes with gold MC-view + defense-depth labels and boundary-teaching notes
  so the 9 teachers can calibrate to kappa>=0.6 before annotating.
</commit_message>
<xml_diff>
--- a/backend/exports/yandaojie/deliverables/packets_validity/packet_数学_T1.xlsx
+++ b/backend/exports/yandaojie/deliverables/packets_validity/packet_数学_T1.xlsx
@@ -8,7 +8,9 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="编码手册" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="标注表" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="评分SOP" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="对齐练习" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="标注表" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -46,6 +48,11 @@
     <font>
       <name val="Arial"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="12"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -132,7 +139,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -175,25 +182,31 @@
     <xf numFmtId="0" fontId="4" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -856,6 +869,619 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:B8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="78" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>评分流程 SOP（标注前必读）</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="16" t="inlineStr">
+        <is>
+          <t>1. 读手册</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>先读「编码手册」sheet，重点记 ②辩护深度 的 5 档定义与 4 条判别规则。</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="16" t="inlineStr">
+        <is>
+          <t>2. 对齐练习(norming)</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>三位老师各自**独立**标完「对齐练习」sheet 的 8 条 → 与主持人手中的 gold key 逐条对照 → 讨论分歧（重点：对标签错机制 vs 空洞、语言科→难判断）→ 统一理解。对齐后再开始正式标注。</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="16" t="inlineStr">
+        <is>
+          <t>3. 正式标注</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>在「标注表」逐行**独立**标注 ①MC视角 ②辩护深度 ③揭示了什么(引用一句) ④信心。三位老师互不商量。</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>原则</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>①只看学生说出的答案；②看整段辩护；二者**独立**。只要追问下机制站不住，就**不算“扎实”**（哪怕答案全对）。信息不足 → 难判断 + 低信心。语言科若无可辩护的机制 → 难判断。</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="17" t="inlineStr">
+        <is>
+          <t>节奏</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>每条约 2–3 分钟；进入下一条后不回改上一条。</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>完成</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>交回文件；研究者计算评分员信度(κ)。若某维度 κ&lt;0.6，回到 norming 再对齐一轮后重标该批。</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="62" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="40" customHeight="1">
+      <c r="A1" s="18" t="inlineStr">
+        <is>
+          <t>序号</t>
+        </is>
+      </c>
+      <c r="B1" s="18" t="inlineStr">
+        <is>
+          <t>学生</t>
+        </is>
+      </c>
+      <c r="C1" s="18" t="inlineStr">
+        <is>
+          <t>课题</t>
+        </is>
+      </c>
+      <c r="D1" s="18" t="inlineStr">
+        <is>
+          <t>本课学习目标</t>
+        </is>
+      </c>
+      <c r="E1" s="18" t="inlineStr">
+        <is>
+          <t>学生反思（输入）</t>
+        </is>
+      </c>
+      <c r="F1" s="18" t="inlineStr">
+        <is>
+          <t>完整辩护对话（AI追问 → 学生作答，逐轮）</t>
+        </is>
+      </c>
+      <c r="G1" s="18" t="inlineStr">
+        <is>
+          <t>①MC视角
+(只看答案/结论)</t>
+        </is>
+      </c>
+      <c r="H1" s="18" t="inlineStr">
+        <is>
+          <t>②辩护深度
+(看完整辩护)</t>
+        </is>
+      </c>
+      <c r="I1" s="18" t="inlineStr">
+        <is>
+          <t>③辩护揭示了什么(引用一句)</t>
+        </is>
+      </c>
+      <c r="J1" s="18" t="inlineStr">
+        <is>
+          <t>④信心(1–5)</t>
+        </is>
+      </c>
+      <c r="K1" s="18" t="inlineStr">
+        <is>
+          <t>评分老师</t>
+        </is>
+      </c>
+      <c r="L1" s="18" t="inlineStr">
+        <is>
+          <t>备注</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="150" customHeight="1">
+      <c r="A2" s="19" t="inlineStr">
+        <is>
+          <t>数6</t>
+        </is>
+      </c>
+      <c r="B2" s="20" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="C2" s="20" t="inlineStr">
+        <is>
+          <t>《可爱的小猫》</t>
+        </is>
+      </c>
+      <c r="D2" s="20" t="inlineStr">
+        <is>
+          <t>1) 经历将“小猫乐乐”在方格纸上利用“数对”放大的探索过程，通过“填一填”“画一画”等活动，体会用“数对”的变化进行图形的放大与缩小的方法，积累数学活动经验。
+2) 在活动中体验图形的多种变化，感受在方格纸上利用“数对”进行图形的放大与缩小的趣味性，激发数学兴趣。</t>
+        </is>
+      </c>
+      <c r="E2" s="20" t="inlineStr">
+        <is>
+          <t>目标1：学到=「数对前后的数同时乘或除以一个相同的数，图形形状不变。」</t>
+        </is>
+      </c>
+      <c r="F2" s="20" t="inlineStr">
+        <is>
+          <t>R1 AI：你在方格纸上放大图形时，具体是怎么改变数对的？请用小猫乐乐的一个点举例说明变化前后的数对。
+    学生：「(0,2)同时乘2得（0，4）」
+R2 AI：你把(0,2)乘2变成了(0,4)，那么小猫的其他点应该怎么变化？请解释原因。
+    学生：「前后同时乘2，因为都乘2，图形不变」
+R3 AI：你刚才说“图形不变”，但放大后的图形应该变大了呀，你觉得这里的“图形不变”是什么意思？
+    学生：「（空）」
+R4 AI：你刚才提到“图形不变”，但放大后的图形大小改变了，为什么还说图形不变呢？请解释一下你的想法。
+    学生：「是图形形状不变」</t>
+        </is>
+      </c>
+      <c r="G2" s="21" t="n"/>
+      <c r="H2" s="21" t="n"/>
+      <c r="I2" s="22" t="n"/>
+      <c r="J2" s="21" t="n"/>
+      <c r="K2" s="23" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="L2" s="24" t="n"/>
+    </row>
+    <row r="3" ht="150" customHeight="1">
+      <c r="A3" s="19" t="inlineStr">
+        <is>
+          <t>数2</t>
+        </is>
+      </c>
+      <c r="B3" s="20" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="C3" s="20" t="inlineStr">
+        <is>
+          <t>《可爱的小猫》</t>
+        </is>
+      </c>
+      <c r="D3" s="20" t="inlineStr">
+        <is>
+          <t>1) 经历将“小猫乐乐”在方格纸上利用“数对”放大的探索过程，通过“填一填”“画一画”等活动，体会用“数对”的变化进行图形的放大与缩小的方法，积累数学活动经验。
+2) 在活动中体验图形的多种变化，感受在方格纸上利用“数对”进行图形的放大与缩小的趣味性，激发数学兴趣。</t>
+        </is>
+      </c>
+      <c r="E3" s="20" t="inlineStr">
+        <is>
+          <t>目标1：学到=「数对里的两个数字同时乘一个不为零的数字与原来图形相向」；疑问=「无」</t>
+        </is>
+      </c>
+      <c r="F3" s="20" t="inlineStr">
+        <is>
+          <t>R1 AI：你说“数对里的两个数字同时乘一个不为零的数字与原来图形相向”，这里的“相向”是指图形形状不变吗？如果我们将小猫乐乐每个点的数对都乘2，画出新图形后，新图形和原图形相比到底发生了什么变化？为什么会这样？
+    学生：「是原图形的每条线段按比例放大到原来的二分之一」
+R2 AI：你刚才说将每个点的数对乘2后，新图形的每条线段按比例放大到原来的二分之一，为什么是二分之一而不是2倍呢？请解释你的想法。
+    学生：「说错了不好意思，是两倍」
+R3 AI：你刚才说乘2后图形变成原来的两倍，那如果想将小猫乐乐缩小到原来的一半，你会如何改变数对？为什么这样做？
+    学生：「将数对的两个数字同时乘二分之一，因为这样会按比例缩小，不影响形状」
+R4 AI：你在反思中提到“乘一个不为零的数字”，如果乘0，会画出什么图形？请解释你的想法。
+    学生：「任何数字乘0都等于0，将两个数字都乘0就没有图形了」
+R4 AI：你刚才说乘0后就没有图形了，但如果所有点都在(0,0)，在方格纸上我们能画出什么？请解释你的想法。
+    学生：「任何数字乘0都等于0，将两个数字都乘0就没有图形了」</t>
+        </is>
+      </c>
+      <c r="G3" s="21" t="n"/>
+      <c r="H3" s="21" t="n"/>
+      <c r="I3" s="22" t="n"/>
+      <c r="J3" s="21" t="n"/>
+      <c r="K3" s="23" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="L3" s="24" t="n"/>
+    </row>
+    <row r="4" ht="150" customHeight="1">
+      <c r="A4" s="19" t="inlineStr">
+        <is>
+          <t>数1</t>
+        </is>
+      </c>
+      <c r="B4" s="20" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="C4" s="20" t="inlineStr">
+        <is>
+          <t>《可爱的小猫》</t>
+        </is>
+      </c>
+      <c r="D4" s="20" t="inlineStr">
+        <is>
+          <t>1) 经历将“小猫乐乐”在方格纸上利用“数对”放大的探索过程，通过“填一填”“画一画”等活动，体会用“数对”的变化进行图形的放大与缩小的方法，积累数学活动经验。
+2) 在活动中体验图形的多种变化，感受在方格纸上利用“数对”进行图形的放大与缩小的趣味性，激发数学兴趣。</t>
+        </is>
+      </c>
+      <c r="E4" s="20" t="inlineStr">
+        <is>
+          <t>目标1：学到=「数对的横轴，纵轴和数对的表示方法」</t>
+        </is>
+      </c>
+      <c r="F4" s="20" t="inlineStr">
+        <is>
+          <t>R1 AI：你已经知道数对可以表示方格纸上的点，如果要把小猫乐乐的图形放大到原来的2倍，你认为每个点的数对应该怎样变化？请解释你的想法。
+    学生：「如果是(2,8),变成（4，16）」
+R2 AI：你提到将数对的两个数都乘以2，这样新的点位置有什么变化？画出的新图形大小和形状会怎样？请解释你的理由。
+    学生：「会向上向右2格，」</t>
+        </is>
+      </c>
+      <c r="G4" s="21" t="n"/>
+      <c r="H4" s="21" t="n"/>
+      <c r="I4" s="22" t="n"/>
+      <c r="J4" s="21" t="n"/>
+      <c r="K4" s="23" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="L4" s="24" t="n"/>
+    </row>
+    <row r="5" ht="150" customHeight="1">
+      <c r="A5" s="19" t="inlineStr">
+        <is>
+          <t>数29</t>
+        </is>
+      </c>
+      <c r="B5" s="20" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="C5" s="20" t="inlineStr">
+        <is>
+          <t>《可爱的小猫》</t>
+        </is>
+      </c>
+      <c r="D5" s="20" t="inlineStr">
+        <is>
+          <t>1) 经历将“小猫乐乐”在方格纸上利用“数对”放大的探索过程，通过“填一填”“画一画”等活动，体会用“数对”的变化进行图形的放大与缩小的方法，积累数学活动经验。
+2) 在活动中体验图形的多种变化，感受在方格纸上利用“数对”进行图形的放大与缩小的趣味性，激发数学兴趣。</t>
+        </is>
+      </c>
+      <c r="E5" s="20" t="inlineStr">
+        <is>
+          <t>目标1：学到=「横轴与纵轴，在数对中横轴与纵轴同时乘或除以一个相同的数（0除外）得到的图形与图形最像。」</t>
+        </is>
+      </c>
+      <c r="F5" s="20" t="inlineStr">
+        <is>
+          <t>R1 AI：你说横轴与纵轴同时乘或除以一个相同的数得到的图形最像，请解释为什么这样做得到的图形会最像呢？
+    学生：「因为当设前项为x，后项为y,」
+R2 AI：你说“因为当设前项为x，后项为y,”，请把你的想法说完，解释为什么横轴和纵轴同时乘或除以相同的数，图形就会最像？
+    学生：「（空）」
+R3 AI：你上次写到“因为当设前项为x，后项为y,”，请以小猫图形上的一个点为例，说明为什么x和y同时乘相同数后，新图形与原图形形状相似？
+    学生：「（空）」
+R3 AI：你刚才说‘当第一项乘一个数，第二项也乘一个相同的数，前后可以约分，就是x，’，请你用一个具体的点，比如小猫身上的点(3,2)，把这句话说完，解释为什么这样做就能让图形形状不变？
+    学生：「（空）」
+R4 AI：你提到“前后可以约分，就是x”，请用小猫身上的点(3,2)为例，把这句话说完，解释把(3,2)的横纵坐标都乘2后，新点(6,4)与原点相比，为什么图形形状不变？
+    学生：「因为6除以2等于3 ，4除以2等于2，他们都是除以一个相同的数得出（3，2）」</t>
+        </is>
+      </c>
+      <c r="G5" s="21" t="n"/>
+      <c r="H5" s="21" t="n"/>
+      <c r="I5" s="22" t="n"/>
+      <c r="J5" s="21" t="n"/>
+      <c r="K5" s="23" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="L5" s="24" t="n"/>
+    </row>
+    <row r="6" ht="150" customHeight="1">
+      <c r="A6" s="19" t="inlineStr">
+        <is>
+          <t>数15</t>
+        </is>
+      </c>
+      <c r="B6" s="20" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C6" s="20" t="inlineStr">
+        <is>
+          <t>《可爱的小猫》</t>
+        </is>
+      </c>
+      <c r="D6" s="20" t="inlineStr">
+        <is>
+          <t>1) 经历将“小猫乐乐”在方格纸上利用“数对”放大的探索过程，通过“填一填”“画一画”等活动，体会用“数对”的变化进行图形的放大与缩小的方法，积累数学活动经验。
+2) 在活动中体验图形的多种变化，感受在方格纸上利用“数对”进行图形的放大与缩小的趣味性，激发数学兴趣。</t>
+        </is>
+      </c>
+      <c r="E6" s="20" t="inlineStr">
+        <is>
+          <t>目标1：学到=「如何观察不同数对
+找数对中不同的规律
+根据规律画出图案」</t>
+        </is>
+      </c>
+      <c r="F6" s="20" t="inlineStr">
+        <is>
+          <t>R1 AI：你提到通过找数对的规律来画出图案，请具体说说，你是怎样从原图数对得到放大的数对的？
+    学生：「观察前后的数找倍数关系」
+R2 AI：你提到“观察前后的数找倍数关系”，请以小猫的一个点为例，具体说说你是怎样用这个倍数关系从原点对得到新点对的？
+    学生：「若前面的数对为（2，3），后面的为（4，6），」
+R3 AI：你举的例子中（4,6）是（2,3）的两倍，那么小猫的其他点是否也都用了相同的两倍关系？请以另一个点为例说明。
+    学生：「有，比如：（3，5）和（6，10）为两倍关系」
+R4 AI：你通过乘以2得到了放大后的数对并画出了新图形，请问画出的放大图与原来的小猫像吗？结合你的画图经验说明理由。
+    学生：「像，因为按照等比例放大或缩小，图形的整体会比较相似。」
+R4 AI：你说等比例放大图形会相似，那么如果要把小猫缩小到原来的一半，数对应该怎么变化？请以（6,10）为例说明。
+    学生：「像，因为按照等比例放大或缩小，图形的整体会比较相似。」</t>
+        </is>
+      </c>
+      <c r="G6" s="21" t="n"/>
+      <c r="H6" s="21" t="n"/>
+      <c r="I6" s="22" t="n"/>
+      <c r="J6" s="21" t="n"/>
+      <c r="K6" s="23" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="L6" s="24" t="n"/>
+    </row>
+    <row r="7" ht="150" customHeight="1">
+      <c r="A7" s="19" t="inlineStr">
+        <is>
+          <t>数24</t>
+        </is>
+      </c>
+      <c r="B7" s="20" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="C7" s="20" t="inlineStr">
+        <is>
+          <t>《可爱的小猫》</t>
+        </is>
+      </c>
+      <c r="D7" s="20" t="inlineStr">
+        <is>
+          <t>1) 经历将“小猫乐乐”在方格纸上利用“数对”放大的探索过程，通过“填一填”“画一画”等活动，体会用“数对”的变化进行图形的放大与缩小的方法，积累数学活动经验。
+2) 在活动中体验图形的多种变化，感受在方格纸上利用“数对”进行图形的放大与缩小的趣味性，激发数学兴趣。</t>
+        </is>
+      </c>
+      <c r="E7" s="20" t="inlineStr">
+        <is>
+          <t>目标1：学到=「数对各点按等比例扩大或缩小才与原图形最像」；疑问=「无」</t>
+        </is>
+      </c>
+      <c r="F7" s="20" t="inlineStr">
+        <is>
+          <t>R1 AI：你提到“数对各点按等比例扩大或缩小才与原图形最像”，那请结合小猫乐乐的某个点，说说你是怎样用数对进行等比例放大的？
+    学生：「例如a点 它对应的数对是（x，y） 必须是（bx，by）」
+R2 AI：你用“(bx, by)”放大了a点，那么小猫乐乐身上其他点的数对也需要乘以同一个b吗？如果b不一样会发生什么？
+    学生：「（空）」
+R3 AI：你在反思中说‘数对各点按等比例扩大或缩小才与原图形最像’，那么如果小猫乐乐的不同点乘以不同的b，图形会变成什么样？请结合你的反思解释一下。
+    学生：「因为第一个数是都乘2 而第二个不是这样」
+R3 AI：你用数对举例说明一下，比如原图有两点A(1,1)和B(1,3)，如果A放大为(2,2)而B放大为(2,5)，它们的边长比例与原图相比怎么不同了？
+    学生：「因为第一个数是都乘2 而第二个不是这样」
+R3 AI：你说第一个数都乘2，第二个不是这样，那么B点的纵坐标从3变成5是乘以了几？这导致竖直边AB的长度比原来扩大了多少倍？
+    学生：「因为第一个数是都乘2 而第二个不是这样」</t>
+        </is>
+      </c>
+      <c r="G7" s="21" t="n"/>
+      <c r="H7" s="21" t="n"/>
+      <c r="I7" s="22" t="n"/>
+      <c r="J7" s="21" t="n"/>
+      <c r="K7" s="23" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="L7" s="24" t="n"/>
+    </row>
+    <row r="8" ht="150" customHeight="1">
+      <c r="A8" s="19" t="inlineStr">
+        <is>
+          <t>科2</t>
+        </is>
+      </c>
+      <c r="B8" s="20" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C8" s="20" t="inlineStr">
+        <is>
+          <t>《厨房里的物质变化》</t>
+        </is>
+      </c>
+      <c r="D8" s="20" t="inlineStr">
+        <is>
+          <t>1) 能列举生活中常见的物理变化（如水结冰、盐溶解）和化学变化（如苹果氧化、铁锅生锈）实例，并用“是否产生新物质”这一核心标准对物质变化进行初步分类。
+2) 通过观察厨房中水、食盐、苹果等物质的状态与特征，运用比较、分析、归纳的方法，自主建构物理变化和化学变化的概念模型。
+3) 能够针对厨房中的特定现象（如切菜、烧水、煎蛋），准确描述其变化前后的特征，并能基于观察提出可探究方法。
+4) 在探究活动中体会科学与生活的紧密联系，感受物质变化的奇妙，初步树立安全用火、合理处理厨余垃圾的生活责任意识。</t>
+        </is>
+      </c>
+      <c r="E8" s="20" t="inlineStr">
+        <is>
+          <t>目标1：学到=「我学到了物质的变化有化学变化也有物理变化，化学变化是产生了新的物质，物理变化是没有产生新物质」</t>
+        </is>
+      </c>
+      <c r="F8" s="20" t="inlineStr">
+        <is>
+          <t>R1 AI：你提到化学变化产生新物质，物理变化没有，那么你能从厨房里找出一个物理变化和一个化学变化的例子，并用这个标准解释为什么这样分类吗？
+    学生：「比如化学变化有鸡蛋从神的变化成sh」
+R2 AI：你提到了鸡蛋从“神”的变化成“sh”，老师不太确定你想说的是不是“生的变成熟的”？请你完整地说一说鸡蛋煮熟的过程是否符合产生新物质的标准，为什么？
+    学生：「（空）」
+R3 AI：你上次说鸡蛋从生的变成熟的，请你现在完整地解释一下：鸡蛋煮熟后有没有产生新物质？为什么？
+    学生：「产生了因为他产生了气味」
+R4 AI：你说鸡蛋煮熟产生了气味，所以觉得产生了新物质。但气味也可能是鸡蛋里原来的物质受热挥发出来的。你怎么判断这个气味是煮的过程里新生成的物质，而不是原来就有的呢？
+    学生：「（空）」
+R5 AI：你还没回答气味是原有的还是新生成的，那换个角度想一想：除了气味，鸡蛋煮熟前后还有什么明显的变化？这些变化能不能说明产生了新物质？
+    学生：「比如它产生了发热和蛋白从变白」</t>
+        </is>
+      </c>
+      <c r="G8" s="21" t="n"/>
+      <c r="H8" s="21" t="n"/>
+      <c r="I8" s="22" t="n"/>
+      <c r="J8" s="21" t="n"/>
+      <c r="K8" s="23" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="L8" s="24" t="n"/>
+    </row>
+    <row r="9" ht="150" customHeight="1">
+      <c r="A9" s="19" t="inlineStr">
+        <is>
+          <t>英20</t>
+        </is>
+      </c>
+      <c r="B9" s="20" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="C9" s="20" t="inlineStr">
+        <is>
+          <t>Unit 6 Summer Vacation</t>
+        </is>
+      </c>
+      <c r="D9" s="20" t="inlineStr">
+        <is>
+          <t>1) 通过听、说、读、写等形式的语言活动，帮助学生复习前几册有关Travel Plan, Winter Vacation, Special Days, Transportation和Around the World等话题的重点词汇和功能句，引导学生综合运用所学语言知识和技能进行交流。
+2) 引导学生就所听材料或所读短文的内容与他人展开对话交流。
+3) 引导学生仿照阅读文段，按相应的提示或要求写几个意义连贯的句子。</t>
+        </is>
+      </c>
+      <c r="E9" s="20" t="inlineStr">
+        <is>
+          <t>目标1：学到=「学到了做暑假计划」</t>
+        </is>
+      </c>
+      <c r="F9" s="20" t="inlineStr">
+        <is>
+          <t>R1 AI：你的暑假计划是什么？请用英语回答。
+    学生：「shanghai」
+R1 AI：你说的“Play”，具体要去哪里玩呢？请用英语回答。
+    学生：「shanghai」
+R2 AI：你在上海具体要做什么？请用英语回答。
+    学生：「play」
+R3 AI：你一直说“play”，能详细说说你在上海打算玩什么娱乐项目或运动吗？请用英语回答。
+    学生：「iat」
+R4 AI：你怎么去上海？请用英语回答。
+    学生：「by plane」</t>
+        </is>
+      </c>
+      <c r="G9" s="21" t="n"/>
+      <c r="H9" s="21" t="n"/>
+      <c r="I9" s="22" t="n"/>
+      <c r="J9" s="21" t="n"/>
+      <c r="K9" s="23" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="L9" s="24" t="n"/>
+    </row>
+  </sheetData>
+  <dataValidations count="3">
+    <dataValidation sqref="G2:G9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"已掌握,部分,未掌握"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H2:H9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"扎实,对标签错机制,空洞或猜对,完全不懂,难判断"</formula1>
+    </dataValidation>
+    <dataValidation sqref="J2:J9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"1,2,3,4,5"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:L32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -874,97 +1500,97 @@
   </cols>
   <sheetData>
     <row r="1" ht="40" customHeight="1">
-      <c r="A1" s="16" t="inlineStr">
+      <c r="A1" s="18" t="inlineStr">
         <is>
           <t>序号</t>
         </is>
       </c>
-      <c r="B1" s="16" t="inlineStr">
+      <c r="B1" s="18" t="inlineStr">
         <is>
           <t>学生</t>
         </is>
       </c>
-      <c r="C1" s="16" t="inlineStr">
+      <c r="C1" s="18" t="inlineStr">
         <is>
           <t>课题</t>
         </is>
       </c>
-      <c r="D1" s="16" t="inlineStr">
+      <c r="D1" s="18" t="inlineStr">
         <is>
           <t>本课学习目标</t>
         </is>
       </c>
-      <c r="E1" s="16" t="inlineStr">
+      <c r="E1" s="18" t="inlineStr">
         <is>
           <t>学生反思（输入）</t>
         </is>
       </c>
-      <c r="F1" s="16" t="inlineStr">
+      <c r="F1" s="18" t="inlineStr">
         <is>
           <t>完整辩护对话（AI追问 → 学生作答，逐轮）</t>
         </is>
       </c>
-      <c r="G1" s="16" t="inlineStr">
+      <c r="G1" s="18" t="inlineStr">
         <is>
           <t>①MC视角
 (只看答案/结论)</t>
         </is>
       </c>
-      <c r="H1" s="16" t="inlineStr">
+      <c r="H1" s="18" t="inlineStr">
         <is>
           <t>②辩护深度
 (看完整辩护)</t>
         </is>
       </c>
-      <c r="I1" s="16" t="inlineStr">
+      <c r="I1" s="18" t="inlineStr">
         <is>
           <t>③辩护揭示了什么(引用一句)</t>
         </is>
       </c>
-      <c r="J1" s="16" t="inlineStr">
+      <c r="J1" s="18" t="inlineStr">
         <is>
           <t>④信心(1–5)</t>
         </is>
       </c>
-      <c r="K1" s="16" t="inlineStr">
+      <c r="K1" s="18" t="inlineStr">
         <is>
           <t>评分老师</t>
         </is>
       </c>
-      <c r="L1" s="16" t="inlineStr">
+      <c r="L1" s="18" t="inlineStr">
         <is>
           <t>备注</t>
         </is>
       </c>
     </row>
     <row r="2" ht="150" customHeight="1">
-      <c r="A2" s="17" t="inlineStr">
+      <c r="A2" s="19" t="inlineStr">
         <is>
           <t>数12</t>
         </is>
       </c>
-      <c r="B2" s="18" t="inlineStr">
+      <c r="B2" s="20" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="C2" s="18" t="inlineStr">
-        <is>
-          <t>《可爱的小猫》</t>
-        </is>
-      </c>
-      <c r="D2" s="18" t="inlineStr">
-        <is>
-          <t>1) 经历将“小猫乐乐”在方格纸上利用“数对”放大的探索过程，通过“填一填”“画一画”等活动，体会用“数对”的变化进行图形的放大与缩小的方法，积累数学活动经验。
-2) 在活动中体验图形的多种变化，感受在方格纸上利用“数对”进行图形的放大与缩小的趣味性，激发数学兴趣。</t>
-        </is>
-      </c>
-      <c r="E2" s="18" t="inlineStr">
+      <c r="C2" s="20" t="inlineStr">
+        <is>
+          <t>《可爱的小猫》</t>
+        </is>
+      </c>
+      <c r="D2" s="20" t="inlineStr">
+        <is>
+          <t>1) 经历将“小猫乐乐”在方格纸上利用“数对”放大的探索过程，通过“填一填”“画一画”等活动，体会用“数对”的变化进行图形的放大与缩小的方法，积累数学活动经验。
+2) 在活动中体验图形的多种变化，感受在方格纸上利用“数对”进行图形的放大与缩小的趣味性，激发数学兴趣。</t>
+        </is>
+      </c>
+      <c r="E2" s="20" t="inlineStr">
         <is>
           <t>目标1：学到=「数对的前面或后面同时乘或除以一个相同的数，画出来的图形才像」；疑问=「无」</t>
         </is>
       </c>
-      <c r="F2" s="18" t="inlineStr">
+      <c r="F2" s="20" t="inlineStr">
         <is>
           <t>R1 AI：你能举个例子说说，为什么数对的两个数都要同时乘或除以相同的数，画出来的图形才像吗？比如把一个三角形的顶点数对（2,1）放大2倍，会变成什么？如果只乘第一个数，图形会怎样？
     学生：「三角形，会变形」
@@ -976,45 +1602,45 @@
     学生：「（空）」</t>
         </is>
       </c>
-      <c r="G2" s="19" t="n"/>
-      <c r="H2" s="19" t="n"/>
-      <c r="I2" s="20" t="n"/>
-      <c r="J2" s="19" t="n"/>
-      <c r="K2" s="21" t="inlineStr">
-        <is>
-          <t>T1</t>
-        </is>
-      </c>
-      <c r="L2" s="22" t="n"/>
+      <c r="G2" s="21" t="n"/>
+      <c r="H2" s="21" t="n"/>
+      <c r="I2" s="22" t="n"/>
+      <c r="J2" s="21" t="n"/>
+      <c r="K2" s="23" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="L2" s="24" t="n"/>
     </row>
     <row r="3" ht="150" customHeight="1">
-      <c r="A3" s="17" t="inlineStr">
+      <c r="A3" s="19" t="inlineStr">
         <is>
           <t>数5</t>
         </is>
       </c>
-      <c r="B3" s="18" t="inlineStr">
+      <c r="B3" s="20" t="inlineStr">
         <is>
           <t>40</t>
         </is>
       </c>
-      <c r="C3" s="18" t="inlineStr">
-        <is>
-          <t>《可爱的小猫》</t>
-        </is>
-      </c>
-      <c r="D3" s="18" t="inlineStr">
-        <is>
-          <t>1) 经历将“小猫乐乐”在方格纸上利用“数对”放大的探索过程，通过“填一填”“画一画”等活动，体会用“数对”的变化进行图形的放大与缩小的方法，积累数学活动经验。
-2) 在活动中体验图形的多种变化，感受在方格纸上利用“数对”进行图形的放大与缩小的趣味性，激发数学兴趣。</t>
-        </is>
-      </c>
-      <c r="E3" s="18" t="inlineStr">
+      <c r="C3" s="20" t="inlineStr">
+        <is>
+          <t>《可爱的小猫》</t>
+        </is>
+      </c>
+      <c r="D3" s="20" t="inlineStr">
+        <is>
+          <t>1) 经历将“小猫乐乐”在方格纸上利用“数对”放大的探索过程，通过“填一填”“画一画”等活动，体会用“数对”的变化进行图形的放大与缩小的方法，积累数学活动经验。
+2) 在活动中体验图形的多种变化，感受在方格纸上利用“数对”进行图形的放大与缩小的趣味性，激发数学兴趣。</t>
+        </is>
+      </c>
+      <c r="E3" s="20" t="inlineStr">
         <is>
           <t>目标1：学到=「数对前后两个数同时乘相同的数，改变后的图形像原来的图形」；疑问=「数对前后两个数同时除以相同的数，改变后的图形像不像原来的图形」</t>
         </is>
       </c>
-      <c r="F3" s="18" t="inlineStr">
+      <c r="F3" s="20" t="inlineStr">
         <is>
           <t>R1 AI：如果试着把小猫乐乐的每个数对都除以2，你认为图形会变成什么样子，为什么？
     学生：「因为每条边都缩小到原来的二分之一」
@@ -1022,45 +1648,45 @@
     学生：「因为每条边都缩小到原来的二分之一」</t>
         </is>
       </c>
-      <c r="G3" s="19" t="n"/>
-      <c r="H3" s="19" t="n"/>
-      <c r="I3" s="20" t="n"/>
-      <c r="J3" s="19" t="n"/>
-      <c r="K3" s="21" t="inlineStr">
-        <is>
-          <t>T1</t>
-        </is>
-      </c>
-      <c r="L3" s="22" t="n"/>
+      <c r="G3" s="21" t="n"/>
+      <c r="H3" s="21" t="n"/>
+      <c r="I3" s="22" t="n"/>
+      <c r="J3" s="21" t="n"/>
+      <c r="K3" s="23" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="L3" s="24" t="n"/>
     </row>
     <row r="4" ht="150" customHeight="1">
-      <c r="A4" s="17" t="inlineStr">
+      <c r="A4" s="19" t="inlineStr">
         <is>
           <t>数14</t>
         </is>
       </c>
-      <c r="B4" s="18" t="inlineStr">
+      <c r="B4" s="20" t="inlineStr">
         <is>
           <t>16</t>
         </is>
       </c>
-      <c r="C4" s="18" t="inlineStr">
-        <is>
-          <t>《可爱的小猫》</t>
-        </is>
-      </c>
-      <c r="D4" s="18" t="inlineStr">
-        <is>
-          <t>1) 经历将“小猫乐乐”在方格纸上利用“数对”放大的探索过程，通过“填一填”“画一画”等活动，体会用“数对”的变化进行图形的放大与缩小的方法，积累数学活动经验。
-2) 在活动中体验图形的多种变化，感受在方格纸上利用“数对”进行图形的放大与缩小的趣味性，激发数学兴趣。</t>
-        </is>
-      </c>
-      <c r="E4" s="18" t="inlineStr">
+      <c r="C4" s="20" t="inlineStr">
+        <is>
+          <t>《可爱的小猫》</t>
+        </is>
+      </c>
+      <c r="D4" s="20" t="inlineStr">
+        <is>
+          <t>1) 经历将“小猫乐乐”在方格纸上利用“数对”放大的探索过程，通过“填一填”“画一画”等活动，体会用“数对”的变化进行图形的放大与缩小的方法，积累数学活动经验。
+2) 在活动中体验图形的多种变化，感受在方格纸上利用“数对”进行图形的放大与缩小的趣味性，激发数学兴趣。</t>
+        </is>
+      </c>
+      <c r="E4" s="20" t="inlineStr">
         <is>
           <t>目标1：学到=「我学到了轮廓上点的位置决定了轮廓的形状位置和大小 以及用数对表示点的位置」</t>
         </is>
       </c>
-      <c r="F4" s="18" t="inlineStr">
+      <c r="F4" s="20" t="inlineStr">
         <is>
           <t>R1 AI：你说轮廓上点的位置决定了形状和大小，那么如果要把一个小猫图形放大，原来点的数对应该怎样变化？请举个例子说明。
     学生：「如果把小猫图形放大2倍 那么横轴和」
@@ -1072,45 +1698,45 @@
     学生：「横轴和竖轴都应放大两倍」</t>
         </is>
       </c>
-      <c r="G4" s="19" t="n"/>
-      <c r="H4" s="19" t="n"/>
-      <c r="I4" s="20" t="n"/>
-      <c r="J4" s="19" t="n"/>
-      <c r="K4" s="21" t="inlineStr">
-        <is>
-          <t>T1</t>
-        </is>
-      </c>
-      <c r="L4" s="22" t="n"/>
+      <c r="G4" s="21" t="n"/>
+      <c r="H4" s="21" t="n"/>
+      <c r="I4" s="22" t="n"/>
+      <c r="J4" s="21" t="n"/>
+      <c r="K4" s="23" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="L4" s="24" t="n"/>
     </row>
     <row r="5" ht="150" customHeight="1">
-      <c r="A5" s="17" t="inlineStr">
+      <c r="A5" s="19" t="inlineStr">
         <is>
           <t>数6</t>
         </is>
       </c>
-      <c r="B5" s="18" t="inlineStr">
+      <c r="B5" s="20" t="inlineStr">
         <is>
           <t>26</t>
         </is>
       </c>
-      <c r="C5" s="18" t="inlineStr">
-        <is>
-          <t>《可爱的小猫》</t>
-        </is>
-      </c>
-      <c r="D5" s="18" t="inlineStr">
-        <is>
-          <t>1) 经历将“小猫乐乐”在方格纸上利用“数对”放大的探索过程，通过“填一填”“画一画”等活动，体会用“数对”的变化进行图形的放大与缩小的方法，积累数学活动经验。
-2) 在活动中体验图形的多种变化，感受在方格纸上利用“数对”进行图形的放大与缩小的趣味性，激发数学兴趣。</t>
-        </is>
-      </c>
-      <c r="E5" s="18" t="inlineStr">
+      <c r="C5" s="20" t="inlineStr">
+        <is>
+          <t>《可爱的小猫》</t>
+        </is>
+      </c>
+      <c r="D5" s="20" t="inlineStr">
+        <is>
+          <t>1) 经历将“小猫乐乐”在方格纸上利用“数对”放大的探索过程，通过“填一填”“画一画”等活动，体会用“数对”的变化进行图形的放大与缩小的方法，积累数学活动经验。
+2) 在活动中体验图形的多种变化，感受在方格纸上利用“数对”进行图形的放大与缩小的趣味性，激发数学兴趣。</t>
+        </is>
+      </c>
+      <c r="E5" s="20" t="inlineStr">
         <is>
           <t>目标1：学到=「数对前后的数同时乘或除以一个相同的数，图形形状不变。」</t>
         </is>
       </c>
-      <c r="F5" s="18" t="inlineStr">
+      <c r="F5" s="20" t="inlineStr">
         <is>
           <t>R1 AI：你在方格纸上放大图形时，具体是怎么改变数对的？请用小猫乐乐的一个点举例说明变化前后的数对。
     学生：「(0,2)同时乘2得（0，4）」
@@ -1122,45 +1748,45 @@
     学生：「是图形形状不变」</t>
         </is>
       </c>
-      <c r="G5" s="19" t="n"/>
-      <c r="H5" s="19" t="n"/>
-      <c r="I5" s="20" t="n"/>
-      <c r="J5" s="19" t="n"/>
-      <c r="K5" s="21" t="inlineStr">
-        <is>
-          <t>T1</t>
-        </is>
-      </c>
-      <c r="L5" s="22" t="n"/>
+      <c r="G5" s="21" t="n"/>
+      <c r="H5" s="21" t="n"/>
+      <c r="I5" s="22" t="n"/>
+      <c r="J5" s="21" t="n"/>
+      <c r="K5" s="23" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="L5" s="24" t="n"/>
     </row>
     <row r="6" ht="150" customHeight="1">
-      <c r="A6" s="17" t="inlineStr">
+      <c r="A6" s="19" t="inlineStr">
         <is>
           <t>数29</t>
         </is>
       </c>
-      <c r="B6" s="18" t="inlineStr">
+      <c r="B6" s="20" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="C6" s="18" t="inlineStr">
-        <is>
-          <t>《可爱的小猫》</t>
-        </is>
-      </c>
-      <c r="D6" s="18" t="inlineStr">
-        <is>
-          <t>1) 经历将“小猫乐乐”在方格纸上利用“数对”放大的探索过程，通过“填一填”“画一画”等活动，体会用“数对”的变化进行图形的放大与缩小的方法，积累数学活动经验。
-2) 在活动中体验图形的多种变化，感受在方格纸上利用“数对”进行图形的放大与缩小的趣味性，激发数学兴趣。</t>
-        </is>
-      </c>
-      <c r="E6" s="18" t="inlineStr">
+      <c r="C6" s="20" t="inlineStr">
+        <is>
+          <t>《可爱的小猫》</t>
+        </is>
+      </c>
+      <c r="D6" s="20" t="inlineStr">
+        <is>
+          <t>1) 经历将“小猫乐乐”在方格纸上利用“数对”放大的探索过程，通过“填一填”“画一画”等活动，体会用“数对”的变化进行图形的放大与缩小的方法，积累数学活动经验。
+2) 在活动中体验图形的多种变化，感受在方格纸上利用“数对”进行图形的放大与缩小的趣味性，激发数学兴趣。</t>
+        </is>
+      </c>
+      <c r="E6" s="20" t="inlineStr">
         <is>
           <t>目标1：学到=「横轴与纵轴，在数对中横轴与纵轴同时乘或除以一个相同的数（0除外）得到的图形与图形最像。」</t>
         </is>
       </c>
-      <c r="F6" s="18" t="inlineStr">
+      <c r="F6" s="20" t="inlineStr">
         <is>
           <t>R1 AI：你说横轴与纵轴同时乘或除以一个相同的数得到的图形最像，请解释为什么这样做得到的图形会最像呢？
     学生：「因为当设前项为x，后项为y,」
@@ -1174,45 +1800,45 @@
     学生：「因为6除以2等于3 ，4除以2等于2，他们都是除以一个相同的数得出（3，2）」</t>
         </is>
       </c>
-      <c r="G6" s="19" t="n"/>
-      <c r="H6" s="19" t="n"/>
-      <c r="I6" s="20" t="n"/>
-      <c r="J6" s="19" t="n"/>
-      <c r="K6" s="21" t="inlineStr">
-        <is>
-          <t>T1</t>
-        </is>
-      </c>
-      <c r="L6" s="22" t="n"/>
+      <c r="G6" s="21" t="n"/>
+      <c r="H6" s="21" t="n"/>
+      <c r="I6" s="22" t="n"/>
+      <c r="J6" s="21" t="n"/>
+      <c r="K6" s="23" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="L6" s="24" t="n"/>
     </row>
     <row r="7" ht="150" customHeight="1">
-      <c r="A7" s="17" t="inlineStr">
+      <c r="A7" s="19" t="inlineStr">
         <is>
           <t>数16</t>
         </is>
       </c>
-      <c r="B7" s="18" t="inlineStr">
+      <c r="B7" s="20" t="inlineStr">
         <is>
           <t>27</t>
         </is>
       </c>
-      <c r="C7" s="18" t="inlineStr">
-        <is>
-          <t>《可爱的小猫》</t>
-        </is>
-      </c>
-      <c r="D7" s="18" t="inlineStr">
-        <is>
-          <t>1) 经历将“小猫乐乐”在方格纸上利用“数对”放大的探索过程，通过“填一填”“画一画”等活动，体会用“数对”的变化进行图形的放大与缩小的方法，积累数学活动经验。
-2) 在活动中体验图形的多种变化，感受在方格纸上利用“数对”进行图形的放大与缩小的趣味性，激发数学兴趣。</t>
-        </is>
-      </c>
-      <c r="E7" s="18" t="inlineStr">
+      <c r="C7" s="20" t="inlineStr">
+        <is>
+          <t>《可爱的小猫》</t>
+        </is>
+      </c>
+      <c r="D7" s="20" t="inlineStr">
+        <is>
+          <t>1) 经历将“小猫乐乐”在方格纸上利用“数对”放大的探索过程，通过“填一填”“画一画”等活动，体会用“数对”的变化进行图形的放大与缩小的方法，积累数学活动经验。
+2) 在活动中体验图形的多种变化，感受在方格纸上利用“数对”进行图形的放大与缩小的趣味性，激发数学兴趣。</t>
+        </is>
+      </c>
+      <c r="E7" s="20" t="inlineStr">
         <is>
           <t>目标1：学到=「掌握数对的前后顺序」</t>
         </is>
       </c>
-      <c r="F7" s="18" t="inlineStr">
+      <c r="F7" s="20" t="inlineStr">
         <is>
           <t>R1 AI：你提到掌握了数对的前后顺序。如果要把方格纸上小猫的一个点放大，比如从(2,1)变成原来的两倍，这个点的数对应该怎么变？请说说你是怎么想的。
     学生：「应该变为（4，2）」
@@ -1222,45 +1848,45 @@
     学生：「它的数对会缩小到（3，4）」</t>
         </is>
       </c>
-      <c r="G7" s="19" t="n"/>
-      <c r="H7" s="19" t="n"/>
-      <c r="I7" s="20" t="n"/>
-      <c r="J7" s="19" t="n"/>
-      <c r="K7" s="21" t="inlineStr">
-        <is>
-          <t>T1</t>
-        </is>
-      </c>
-      <c r="L7" s="22" t="n"/>
+      <c r="G7" s="21" t="n"/>
+      <c r="H7" s="21" t="n"/>
+      <c r="I7" s="22" t="n"/>
+      <c r="J7" s="21" t="n"/>
+      <c r="K7" s="23" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="L7" s="24" t="n"/>
     </row>
     <row r="8" ht="150" customHeight="1">
-      <c r="A8" s="17" t="inlineStr">
+      <c r="A8" s="19" t="inlineStr">
         <is>
           <t>数23</t>
         </is>
       </c>
-      <c r="B8" s="18" t="inlineStr">
+      <c r="B8" s="20" t="inlineStr">
         <is>
           <t>13</t>
         </is>
       </c>
-      <c r="C8" s="18" t="inlineStr">
-        <is>
-          <t>《可爱的小猫》</t>
-        </is>
-      </c>
-      <c r="D8" s="18" t="inlineStr">
-        <is>
-          <t>1) 经历将“小猫乐乐”在方格纸上利用“数对”放大的探索过程，通过“填一填”“画一画”等活动，体会用“数对”的变化进行图形的放大与缩小的方法，积累数学活动经验。
-2) 在活动中体验图形的多种变化，感受在方格纸上利用“数对”进行图形的放大与缩小的趣味性，激发数学兴趣。</t>
-        </is>
-      </c>
-      <c r="E8" s="18" t="inlineStr">
+      <c r="C8" s="20" t="inlineStr">
+        <is>
+          <t>《可爱的小猫》</t>
+        </is>
+      </c>
+      <c r="D8" s="20" t="inlineStr">
+        <is>
+          <t>1) 经历将“小猫乐乐”在方格纸上利用“数对”放大的探索过程，通过“填一填”“画一画”等活动，体会用“数对”的变化进行图形的放大与缩小的方法，积累数学活动经验。
+2) 在活动中体验图形的多种变化，感受在方格纸上利用“数对”进行图形的放大与缩小的趣味性，激发数学兴趣。</t>
+        </is>
+      </c>
+      <c r="E8" s="20" t="inlineStr">
         <is>
           <t>目标1：学到=「数对表达」</t>
         </is>
       </c>
-      <c r="F8" s="18" t="inlineStr">
+      <c r="F8" s="20" t="inlineStr">
         <is>
           <t>R1 AI：你提到学习了数对表达，如果要把小猫乐乐的一个点，比如在数对(2,3)的位置，进行放大，你准备怎么改变这个数对？为什么这样改？
     学生：「（4，6）（8，12）.......」
@@ -1274,45 +1900,45 @@
     学生：「比如（1，2）的长方形如果Y*2」</t>
         </is>
       </c>
-      <c r="G8" s="19" t="n"/>
-      <c r="H8" s="19" t="n"/>
-      <c r="I8" s="20" t="n"/>
-      <c r="J8" s="19" t="n"/>
-      <c r="K8" s="21" t="inlineStr">
-        <is>
-          <t>T1</t>
-        </is>
-      </c>
-      <c r="L8" s="22" t="n"/>
+      <c r="G8" s="21" t="n"/>
+      <c r="H8" s="21" t="n"/>
+      <c r="I8" s="22" t="n"/>
+      <c r="J8" s="21" t="n"/>
+      <c r="K8" s="23" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="L8" s="24" t="n"/>
     </row>
     <row r="9" ht="150" customHeight="1">
-      <c r="A9" s="17" t="inlineStr">
+      <c r="A9" s="19" t="inlineStr">
         <is>
           <t>数2</t>
         </is>
       </c>
-      <c r="B9" s="18" t="inlineStr">
+      <c r="B9" s="20" t="inlineStr">
         <is>
           <t>36</t>
         </is>
       </c>
-      <c r="C9" s="18" t="inlineStr">
-        <is>
-          <t>《可爱的小猫》</t>
-        </is>
-      </c>
-      <c r="D9" s="18" t="inlineStr">
-        <is>
-          <t>1) 经历将“小猫乐乐”在方格纸上利用“数对”放大的探索过程，通过“填一填”“画一画”等活动，体会用“数对”的变化进行图形的放大与缩小的方法，积累数学活动经验。
-2) 在活动中体验图形的多种变化，感受在方格纸上利用“数对”进行图形的放大与缩小的趣味性，激发数学兴趣。</t>
-        </is>
-      </c>
-      <c r="E9" s="18" t="inlineStr">
+      <c r="C9" s="20" t="inlineStr">
+        <is>
+          <t>《可爱的小猫》</t>
+        </is>
+      </c>
+      <c r="D9" s="20" t="inlineStr">
+        <is>
+          <t>1) 经历将“小猫乐乐”在方格纸上利用“数对”放大的探索过程，通过“填一填”“画一画”等活动，体会用“数对”的变化进行图形的放大与缩小的方法，积累数学活动经验。
+2) 在活动中体验图形的多种变化，感受在方格纸上利用“数对”进行图形的放大与缩小的趣味性，激发数学兴趣。</t>
+        </is>
+      </c>
+      <c r="E9" s="20" t="inlineStr">
         <is>
           <t>目标1：学到=「数对里的两个数字同时乘一个不为零的数字与原来图形相向」；疑问=「无」</t>
         </is>
       </c>
-      <c r="F9" s="18" t="inlineStr">
+      <c r="F9" s="20" t="inlineStr">
         <is>
           <t>R1 AI：你说“数对里的两个数字同时乘一个不为零的数字与原来图形相向”，这里的“相向”是指图形形状不变吗？如果我们将小猫乐乐每个点的数对都乘2，画出新图形后，新图形和原图形相比到底发生了什么变化？为什么会这样？
     学生：「是原图形的每条线段按比例放大到原来的二分之一」
@@ -1326,45 +1952,45 @@
     学生：「任何数字乘0都等于0，将两个数字都乘0就没有图形了」</t>
         </is>
       </c>
-      <c r="G9" s="19" t="n"/>
-      <c r="H9" s="19" t="n"/>
-      <c r="I9" s="20" t="n"/>
-      <c r="J9" s="19" t="n"/>
-      <c r="K9" s="21" t="inlineStr">
-        <is>
-          <t>T1</t>
-        </is>
-      </c>
-      <c r="L9" s="22" t="n"/>
+      <c r="G9" s="21" t="n"/>
+      <c r="H9" s="21" t="n"/>
+      <c r="I9" s="22" t="n"/>
+      <c r="J9" s="21" t="n"/>
+      <c r="K9" s="23" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="L9" s="24" t="n"/>
     </row>
     <row r="10" ht="150" customHeight="1">
-      <c r="A10" s="17" t="inlineStr">
+      <c r="A10" s="19" t="inlineStr">
         <is>
           <t>数8</t>
         </is>
       </c>
-      <c r="B10" s="18" t="inlineStr">
+      <c r="B10" s="20" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="C10" s="18" t="inlineStr">
-        <is>
-          <t>《可爱的小猫》</t>
-        </is>
-      </c>
-      <c r="D10" s="18" t="inlineStr">
-        <is>
-          <t>1) 经历将“小猫乐乐”在方格纸上利用“数对”放大的探索过程，通过“填一填”“画一画”等活动，体会用“数对”的变化进行图形的放大与缩小的方法，积累数学活动经验。
-2) 在活动中体验图形的多种变化，感受在方格纸上利用“数对”进行图形的放大与缩小的趣味性，激发数学兴趣。</t>
-        </is>
-      </c>
-      <c r="E10" s="18" t="inlineStr">
+      <c r="C10" s="20" t="inlineStr">
+        <is>
+          <t>《可爱的小猫》</t>
+        </is>
+      </c>
+      <c r="D10" s="20" t="inlineStr">
+        <is>
+          <t>1) 经历将“小猫乐乐”在方格纸上利用“数对”放大的探索过程，通过“填一填”“画一画”等活动，体会用“数对”的变化进行图形的放大与缩小的方法，积累数学活动经验。
+2) 在活动中体验图形的多种变化，感受在方格纸上利用“数对”进行图形的放大与缩小的趣味性，激发数学兴趣。</t>
+        </is>
+      </c>
+      <c r="E10" s="20" t="inlineStr">
         <is>
           <t>目标1：学到=「在一个数对中，横纵坐标同时乘或除以一个相同的数（零除外），得到的图形与原图形像。」</t>
         </is>
       </c>
-      <c r="F10" s="18" t="inlineStr">
+      <c r="F10" s="20" t="inlineStr">
         <is>
           <t>R1 AI：你能解释为什么数对中横纵坐标同时乘相同的数，图形就和原图形像，并用小猫乐乐举例吗？
     学生：「可以画出乐乐，然后画出一个横坐标乘2和纵坐标」
@@ -1378,45 +2004,45 @@
     学生：「因为横纵坐标同时乘2，横轴和纵轴的点会在同一条直线上」</t>
         </is>
       </c>
-      <c r="G10" s="19" t="n"/>
-      <c r="H10" s="19" t="n"/>
-      <c r="I10" s="20" t="n"/>
-      <c r="J10" s="19" t="n"/>
-      <c r="K10" s="21" t="inlineStr">
-        <is>
-          <t>T1</t>
-        </is>
-      </c>
-      <c r="L10" s="22" t="n"/>
+      <c r="G10" s="21" t="n"/>
+      <c r="H10" s="21" t="n"/>
+      <c r="I10" s="22" t="n"/>
+      <c r="J10" s="21" t="n"/>
+      <c r="K10" s="23" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="L10" s="24" t="n"/>
     </row>
     <row r="11" ht="150" customHeight="1">
-      <c r="A11" s="17" t="inlineStr">
+      <c r="A11" s="19" t="inlineStr">
         <is>
           <t>数9</t>
         </is>
       </c>
-      <c r="B11" s="18" t="inlineStr">
+      <c r="B11" s="20" t="inlineStr">
         <is>
           <t>43</t>
         </is>
       </c>
-      <c r="C11" s="18" t="inlineStr">
-        <is>
-          <t>《可爱的小猫》</t>
-        </is>
-      </c>
-      <c r="D11" s="18" t="inlineStr">
-        <is>
-          <t>1) 经历将“小猫乐乐”在方格纸上利用“数对”放大的探索过程，通过“填一填”“画一画”等活动，体会用“数对”的变化进行图形的放大与缩小的方法，积累数学活动经验。
-2) 在活动中体验图形的多种变化，感受在方格纸上利用“数对”进行图形的放大与缩小的趣味性，激发数学兴趣。</t>
-        </is>
-      </c>
-      <c r="E11" s="18" t="inlineStr">
+      <c r="C11" s="20" t="inlineStr">
+        <is>
+          <t>《可爱的小猫》</t>
+        </is>
+      </c>
+      <c r="D11" s="20" t="inlineStr">
+        <is>
+          <t>1) 经历将“小猫乐乐”在方格纸上利用“数对”放大的探索过程，通过“填一填”“画一画”等活动，体会用“数对”的变化进行图形的放大与缩小的方法，积累数学活动经验。
+2) 在活动中体验图形的多种变化，感受在方格纸上利用“数对”进行图形的放大与缩小的趣味性，激发数学兴趣。</t>
+        </is>
+      </c>
+      <c r="E11" s="20" t="inlineStr">
         <is>
           <t>目标1：学到=「我学会了找数对的规律」</t>
         </is>
       </c>
-      <c r="F11" s="18" t="inlineStr">
+      <c r="F11" s="20" t="inlineStr">
         <is>
           <t>R1 AI：你说学会了找数对的规律，能具体说说你是怎样利用这些规律把小猫乐乐的图形放大的吗？
     学生：「根据一个数对之间的关系来放大例如2x2y」
@@ -1426,45 +2052,45 @@
     学生：「2a 2b」</t>
         </is>
       </c>
-      <c r="G11" s="19" t="n"/>
-      <c r="H11" s="19" t="n"/>
-      <c r="I11" s="20" t="n"/>
-      <c r="J11" s="19" t="n"/>
-      <c r="K11" s="21" t="inlineStr">
-        <is>
-          <t>T1</t>
-        </is>
-      </c>
-      <c r="L11" s="22" t="n"/>
+      <c r="G11" s="21" t="n"/>
+      <c r="H11" s="21" t="n"/>
+      <c r="I11" s="22" t="n"/>
+      <c r="J11" s="21" t="n"/>
+      <c r="K11" s="23" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="L11" s="24" t="n"/>
     </row>
     <row r="12" ht="150" customHeight="1">
-      <c r="A12" s="17" t="inlineStr">
+      <c r="A12" s="19" t="inlineStr">
         <is>
           <t>数7</t>
         </is>
       </c>
-      <c r="B12" s="18" t="inlineStr">
+      <c r="B12" s="20" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
-      <c r="C12" s="18" t="inlineStr">
-        <is>
-          <t>《可爱的小猫》</t>
-        </is>
-      </c>
-      <c r="D12" s="18" t="inlineStr">
-        <is>
-          <t>1) 经历将“小猫乐乐”在方格纸上利用“数对”放大的探索过程，通过“填一填”“画一画”等活动，体会用“数对”的变化进行图形的放大与缩小的方法，积累数学活动经验。
-2) 在活动中体验图形的多种变化，感受在方格纸上利用“数对”进行图形的放大与缩小的趣味性，激发数学兴趣。</t>
-        </is>
-      </c>
-      <c r="E12" s="18" t="inlineStr">
+      <c r="C12" s="20" t="inlineStr">
+        <is>
+          <t>《可爱的小猫》</t>
+        </is>
+      </c>
+      <c r="D12" s="20" t="inlineStr">
+        <is>
+          <t>1) 经历将“小猫乐乐”在方格纸上利用“数对”放大的探索过程，通过“填一填”“画一画”等活动，体会用“数对”的变化进行图形的放大与缩小的方法，积累数学活动经验。
+2) 在活动中体验图形的多种变化，感受在方格纸上利用“数对”进行图形的放大与缩小的趣味性，激发数学兴趣。</t>
+        </is>
+      </c>
+      <c r="E12" s="20" t="inlineStr">
         <is>
           <t>目标1：学到=「用点定位」</t>
         </is>
       </c>
-      <c r="F12" s="18" t="inlineStr">
+      <c r="F12" s="20" t="inlineStr">
         <is>
           <t>R1 AI：你提到‘用点定位’，那么怎样用数对表示小猫乐乐图上某个点的位置呢？
     学生：「纵向写1」
@@ -1478,45 +2104,45 @@
     学生：「1排4列的交点」</t>
         </is>
       </c>
-      <c r="G12" s="19" t="n"/>
-      <c r="H12" s="19" t="n"/>
-      <c r="I12" s="20" t="n"/>
-      <c r="J12" s="19" t="n"/>
-      <c r="K12" s="21" t="inlineStr">
-        <is>
-          <t>T1</t>
-        </is>
-      </c>
-      <c r="L12" s="22" t="n"/>
+      <c r="G12" s="21" t="n"/>
+      <c r="H12" s="21" t="n"/>
+      <c r="I12" s="22" t="n"/>
+      <c r="J12" s="21" t="n"/>
+      <c r="K12" s="23" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="L12" s="24" t="n"/>
     </row>
     <row r="13" ht="150" customHeight="1">
-      <c r="A13" s="17" t="inlineStr">
+      <c r="A13" s="19" t="inlineStr">
         <is>
           <t>数24</t>
         </is>
       </c>
-      <c r="B13" s="18" t="inlineStr">
+      <c r="B13" s="20" t="inlineStr">
         <is>
           <t>39</t>
         </is>
       </c>
-      <c r="C13" s="18" t="inlineStr">
-        <is>
-          <t>《可爱的小猫》</t>
-        </is>
-      </c>
-      <c r="D13" s="18" t="inlineStr">
-        <is>
-          <t>1) 经历将“小猫乐乐”在方格纸上利用“数对”放大的探索过程，通过“填一填”“画一画”等活动，体会用“数对”的变化进行图形的放大与缩小的方法，积累数学活动经验。
-2) 在活动中体验图形的多种变化，感受在方格纸上利用“数对”进行图形的放大与缩小的趣味性，激发数学兴趣。</t>
-        </is>
-      </c>
-      <c r="E13" s="18" t="inlineStr">
+      <c r="C13" s="20" t="inlineStr">
+        <is>
+          <t>《可爱的小猫》</t>
+        </is>
+      </c>
+      <c r="D13" s="20" t="inlineStr">
+        <is>
+          <t>1) 经历将“小猫乐乐”在方格纸上利用“数对”放大的探索过程，通过“填一填”“画一画”等活动，体会用“数对”的变化进行图形的放大与缩小的方法，积累数学活动经验。
+2) 在活动中体验图形的多种变化，感受在方格纸上利用“数对”进行图形的放大与缩小的趣味性，激发数学兴趣。</t>
+        </is>
+      </c>
+      <c r="E13" s="20" t="inlineStr">
         <is>
           <t>目标1：学到=「数对各点按等比例扩大或缩小才与原图形最像」；疑问=「无」</t>
         </is>
       </c>
-      <c r="F13" s="18" t="inlineStr">
+      <c r="F13" s="20" t="inlineStr">
         <is>
           <t>R1 AI：你提到“数对各点按等比例扩大或缩小才与原图形最像”，那请结合小猫乐乐的某个点，说说你是怎样用数对进行等比例放大的？
     学生：「例如a点 它对应的数对是（x，y） 必须是（bx，by）」
@@ -1530,45 +2156,45 @@
     学生：「因为第一个数是都乘2 而第二个不是这样」</t>
         </is>
       </c>
-      <c r="G13" s="19" t="n"/>
-      <c r="H13" s="19" t="n"/>
-      <c r="I13" s="20" t="n"/>
-      <c r="J13" s="19" t="n"/>
-      <c r="K13" s="21" t="inlineStr">
-        <is>
-          <t>T1</t>
-        </is>
-      </c>
-      <c r="L13" s="22" t="n"/>
+      <c r="G13" s="21" t="n"/>
+      <c r="H13" s="21" t="n"/>
+      <c r="I13" s="22" t="n"/>
+      <c r="J13" s="21" t="n"/>
+      <c r="K13" s="23" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="L13" s="24" t="n"/>
     </row>
     <row r="14" ht="150" customHeight="1">
-      <c r="A14" s="17" t="inlineStr">
+      <c r="A14" s="19" t="inlineStr">
         <is>
           <t>数27</t>
         </is>
       </c>
-      <c r="B14" s="18" t="inlineStr">
+      <c r="B14" s="20" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="C14" s="18" t="inlineStr">
-        <is>
-          <t>《可爱的小猫》</t>
-        </is>
-      </c>
-      <c r="D14" s="18" t="inlineStr">
-        <is>
-          <t>1) 经历将“小猫乐乐”在方格纸上利用“数对”放大的探索过程，通过“填一填”“画一画”等活动，体会用“数对”的变化进行图形的放大与缩小的方法，积累数学活动经验。
-2) 在活动中体验图形的多种变化，感受在方格纸上利用“数对”进行图形的放大与缩小的趣味性，激发数学兴趣。</t>
-        </is>
-      </c>
-      <c r="E14" s="18" t="inlineStr">
+      <c r="C14" s="20" t="inlineStr">
+        <is>
+          <t>《可爱的小猫》</t>
+        </is>
+      </c>
+      <c r="D14" s="20" t="inlineStr">
+        <is>
+          <t>1) 经历将“小猫乐乐”在方格纸上利用“数对”放大的探索过程，通过“填一填”“画一画”等活动，体会用“数对”的变化进行图形的放大与缩小的方法，积累数学活动经验。
+2) 在活动中体验图形的多种变化，感受在方格纸上利用“数对”进行图形的放大与缩小的趣味性，激发数学兴趣。</t>
+        </is>
+      </c>
+      <c r="E14" s="20" t="inlineStr">
         <is>
           <t>目标1：学到=「如何观察图中的数对，并通过规律改变数对来让他变形」</t>
         </is>
       </c>
-      <c r="F14" s="18" t="inlineStr">
+      <c r="F14" s="20" t="inlineStr">
         <is>
           <t>R1 AI：你能不能结合小猫乐乐的例子，解释一下你学到的通过改变数对让图形变大的规律？
     学生：「让每个点同时乘或除以一个不为0的数来变大」
@@ -1582,45 +2208,45 @@
     学生：「（空）」</t>
         </is>
       </c>
-      <c r="G14" s="19" t="n"/>
-      <c r="H14" s="19" t="n"/>
-      <c r="I14" s="20" t="n"/>
-      <c r="J14" s="19" t="n"/>
-      <c r="K14" s="21" t="inlineStr">
-        <is>
-          <t>T1</t>
-        </is>
-      </c>
-      <c r="L14" s="22" t="n"/>
+      <c r="G14" s="21" t="n"/>
+      <c r="H14" s="21" t="n"/>
+      <c r="I14" s="22" t="n"/>
+      <c r="J14" s="21" t="n"/>
+      <c r="K14" s="23" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="L14" s="24" t="n"/>
     </row>
     <row r="15" ht="150" customHeight="1">
-      <c r="A15" s="17" t="inlineStr">
+      <c r="A15" s="19" t="inlineStr">
         <is>
           <t>数25</t>
         </is>
       </c>
-      <c r="B15" s="18" t="inlineStr">
+      <c r="B15" s="20" t="inlineStr">
         <is>
           <t>4号</t>
         </is>
       </c>
-      <c r="C15" s="18" t="inlineStr">
-        <is>
-          <t>《可爱的小猫》</t>
-        </is>
-      </c>
-      <c r="D15" s="18" t="inlineStr">
-        <is>
-          <t>1) 经历将“小猫乐乐”在方格纸上利用“数对”放大的探索过程，通过“填一填”“画一画”等活动，体会用“数对”的变化进行图形的放大与缩小的方法，积累数学活动经验。
-2) 在活动中体验图形的多种变化，感受在方格纸上利用“数对”进行图形的放大与缩小的趣味性，激发数学兴趣。</t>
-        </is>
-      </c>
-      <c r="E15" s="18" t="inlineStr">
+      <c r="C15" s="20" t="inlineStr">
+        <is>
+          <t>《可爱的小猫》</t>
+        </is>
+      </c>
+      <c r="D15" s="20" t="inlineStr">
+        <is>
+          <t>1) 经历将“小猫乐乐”在方格纸上利用“数对”放大的探索过程，通过“填一填”“画一画”等活动，体会用“数对”的变化进行图形的放大与缩小的方法，积累数学活动经验。
+2) 在活动中体验图形的多种变化，感受在方格纸上利用“数对”进行图形的放大与缩小的趣味性，激发数学兴趣。</t>
+        </is>
+      </c>
+      <c r="E15" s="20" t="inlineStr">
         <is>
           <t>目标1：学到=「数对是如何表示的」</t>
         </is>
       </c>
-      <c r="F15" s="18" t="inlineStr">
+      <c r="F15" s="20" t="inlineStr">
         <is>
           <t>R1 AI：你已经知道数对是如何表示的，那么如果我们要在方格纸上将小猫的图形放大，你猜猜看数对会发生怎样的变化呢？请解释你的想法。
     学生：「数对会变大」
@@ -1630,45 +2256,45 @@
     学生：「因为它要等比例放大」</t>
         </is>
       </c>
-      <c r="G15" s="19" t="n"/>
-      <c r="H15" s="19" t="n"/>
-      <c r="I15" s="20" t="n"/>
-      <c r="J15" s="19" t="n"/>
-      <c r="K15" s="21" t="inlineStr">
-        <is>
-          <t>T1</t>
-        </is>
-      </c>
-      <c r="L15" s="22" t="n"/>
+      <c r="G15" s="21" t="n"/>
+      <c r="H15" s="21" t="n"/>
+      <c r="I15" s="22" t="n"/>
+      <c r="J15" s="21" t="n"/>
+      <c r="K15" s="23" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="L15" s="24" t="n"/>
     </row>
     <row r="16" ht="150" customHeight="1">
-      <c r="A16" s="17" t="inlineStr">
+      <c r="A16" s="19" t="inlineStr">
         <is>
           <t>数3</t>
         </is>
       </c>
-      <c r="B16" s="18" t="inlineStr">
+      <c r="B16" s="20" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="C16" s="18" t="inlineStr">
-        <is>
-          <t>《可爱的小猫》</t>
-        </is>
-      </c>
-      <c r="D16" s="18" t="inlineStr">
-        <is>
-          <t>1) 经历将“小猫乐乐”在方格纸上利用“数对”放大的探索过程，通过“填一填”“画一画”等活动，体会用“数对”的变化进行图形的放大与缩小的方法，积累数学活动经验。
-2) 在活动中体验图形的多种变化，感受在方格纸上利用“数对”进行图形的放大与缩小的趣味性，激发数学兴趣。</t>
-        </is>
-      </c>
-      <c r="E16" s="18" t="inlineStr">
+      <c r="C16" s="20" t="inlineStr">
+        <is>
+          <t>《可爱的小猫》</t>
+        </is>
+      </c>
+      <c r="D16" s="20" t="inlineStr">
+        <is>
+          <t>1) 经历将“小猫乐乐”在方格纸上利用“数对”放大的探索过程，通过“填一填”“画一画”等活动，体会用“数对”的变化进行图形的放大与缩小的方法，积累数学活动经验。
+2) 在活动中体验图形的多种变化，感受在方格纸上利用“数对”进行图形的放大与缩小的趣味性，激发数学兴趣。</t>
+        </is>
+      </c>
+      <c r="E16" s="20" t="inlineStr">
         <is>
           <t>目标1：学到=「数对」；疑问=「数对是谁发明的」</t>
         </is>
       </c>
-      <c r="F16" s="18" t="inlineStr">
+      <c r="F16" s="20" t="inlineStr">
         <is>
           <t>R1 AI：你刚提到了数对，那么在方格纸上，数对（比如(3,2)）里的第一个数和第二个数分别表示什么意思呢？
     学生：「3是第三列2是第
@@ -1683,45 +2309,45 @@
     学生：「2倍」</t>
         </is>
       </c>
-      <c r="G16" s="19" t="n"/>
-      <c r="H16" s="19" t="n"/>
-      <c r="I16" s="20" t="n"/>
-      <c r="J16" s="19" t="n"/>
-      <c r="K16" s="21" t="inlineStr">
-        <is>
-          <t>T1</t>
-        </is>
-      </c>
-      <c r="L16" s="22" t="n"/>
+      <c r="G16" s="21" t="n"/>
+      <c r="H16" s="21" t="n"/>
+      <c r="I16" s="22" t="n"/>
+      <c r="J16" s="21" t="n"/>
+      <c r="K16" s="23" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="L16" s="24" t="n"/>
     </row>
     <row r="17" ht="150" customHeight="1">
-      <c r="A17" s="17" t="inlineStr">
+      <c r="A17" s="19" t="inlineStr">
         <is>
           <t>数30</t>
         </is>
       </c>
-      <c r="B17" s="18" t="inlineStr">
+      <c r="B17" s="20" t="inlineStr">
         <is>
           <t>23</t>
         </is>
       </c>
-      <c r="C17" s="18" t="inlineStr">
-        <is>
-          <t>《可爱的小猫》</t>
-        </is>
-      </c>
-      <c r="D17" s="18" t="inlineStr">
-        <is>
-          <t>1) 经历将“小猫乐乐”在方格纸上利用“数对”放大的探索过程，通过“填一填”“画一画”等活动，体会用“数对”的变化进行图形的放大与缩小的方法，积累数学活动经验。
-2) 在活动中体验图形的多种变化，感受在方格纸上利用“数对”进行图形的放大与缩小的趣味性，激发数学兴趣。</t>
-        </is>
-      </c>
-      <c r="E17" s="18" t="inlineStr">
+      <c r="C17" s="20" t="inlineStr">
+        <is>
+          <t>《可爱的小猫》</t>
+        </is>
+      </c>
+      <c r="D17" s="20" t="inlineStr">
+        <is>
+          <t>1) 经历将“小猫乐乐”在方格纸上利用“数对”放大的探索过程，通过“填一填”“画一画”等活动，体会用“数对”的变化进行图形的放大与缩小的方法，积累数学活动经验。
+2) 在活动中体验图形的多种变化，感受在方格纸上利用“数对”进行图形的放大与缩小的趣味性，激发数学兴趣。</t>
+        </is>
+      </c>
+      <c r="E17" s="20" t="inlineStr">
         <is>
           <t>目标1：学到=「如何用数对绘图」</t>
         </is>
       </c>
-      <c r="F17" s="18" t="inlineStr">
+      <c r="F17" s="20" t="inlineStr">
         <is>
           <t>R1 AI：你说你学会了用数对绘图，如果要让小猫乐乐在方格纸上放大到原来的两倍，它的每个点的数对应该怎么变化呢？请解释。
     学生：「将数对的左右两边都」
@@ -1733,47 +2359,47 @@
     学生：「因为他们都乘了2」</t>
         </is>
       </c>
-      <c r="G17" s="19" t="n"/>
-      <c r="H17" s="19" t="n"/>
-      <c r="I17" s="20" t="n"/>
-      <c r="J17" s="19" t="n"/>
-      <c r="K17" s="21" t="inlineStr">
-        <is>
-          <t>T1</t>
-        </is>
-      </c>
-      <c r="L17" s="22" t="n"/>
+      <c r="G17" s="21" t="n"/>
+      <c r="H17" s="21" t="n"/>
+      <c r="I17" s="22" t="n"/>
+      <c r="J17" s="21" t="n"/>
+      <c r="K17" s="23" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="L17" s="24" t="n"/>
     </row>
     <row r="18" ht="150" customHeight="1">
-      <c r="A18" s="17" t="inlineStr">
+      <c r="A18" s="19" t="inlineStr">
         <is>
           <t>数15</t>
         </is>
       </c>
-      <c r="B18" s="18" t="inlineStr">
+      <c r="B18" s="20" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="C18" s="18" t="inlineStr">
-        <is>
-          <t>《可爱的小猫》</t>
-        </is>
-      </c>
-      <c r="D18" s="18" t="inlineStr">
-        <is>
-          <t>1) 经历将“小猫乐乐”在方格纸上利用“数对”放大的探索过程，通过“填一填”“画一画”等活动，体会用“数对”的变化进行图形的放大与缩小的方法，积累数学活动经验。
-2) 在活动中体验图形的多种变化，感受在方格纸上利用“数对”进行图形的放大与缩小的趣味性，激发数学兴趣。</t>
-        </is>
-      </c>
-      <c r="E18" s="18" t="inlineStr">
+      <c r="C18" s="20" t="inlineStr">
+        <is>
+          <t>《可爱的小猫》</t>
+        </is>
+      </c>
+      <c r="D18" s="20" t="inlineStr">
+        <is>
+          <t>1) 经历将“小猫乐乐”在方格纸上利用“数对”放大的探索过程，通过“填一填”“画一画”等活动，体会用“数对”的变化进行图形的放大与缩小的方法，积累数学活动经验。
+2) 在活动中体验图形的多种变化，感受在方格纸上利用“数对”进行图形的放大与缩小的趣味性，激发数学兴趣。</t>
+        </is>
+      </c>
+      <c r="E18" s="20" t="inlineStr">
         <is>
           <t>目标1：学到=「如何观察不同数对
 找数对中不同的规律
 根据规律画出图案」</t>
         </is>
       </c>
-      <c r="F18" s="18" t="inlineStr">
+      <c r="F18" s="20" t="inlineStr">
         <is>
           <t>R1 AI：你提到通过找数对的规律来画出图案，请具体说说，你是怎样从原图数对得到放大的数对的？
     学生：「观察前后的数找倍数关系」
@@ -1787,45 +2413,45 @@
     学生：「像，因为按照等比例放大或缩小，图形的整体会比较相似。」</t>
         </is>
       </c>
-      <c r="G18" s="19" t="n"/>
-      <c r="H18" s="19" t="n"/>
-      <c r="I18" s="20" t="n"/>
-      <c r="J18" s="19" t="n"/>
-      <c r="K18" s="21" t="inlineStr">
-        <is>
-          <t>T1</t>
-        </is>
-      </c>
-      <c r="L18" s="22" t="n"/>
+      <c r="G18" s="21" t="n"/>
+      <c r="H18" s="21" t="n"/>
+      <c r="I18" s="22" t="n"/>
+      <c r="J18" s="21" t="n"/>
+      <c r="K18" s="23" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="L18" s="24" t="n"/>
     </row>
     <row r="19" ht="150" customHeight="1">
-      <c r="A19" s="17" t="inlineStr">
+      <c r="A19" s="19" t="inlineStr">
         <is>
           <t>数19</t>
         </is>
       </c>
-      <c r="B19" s="18" t="inlineStr">
+      <c r="B19" s="20" t="inlineStr">
         <is>
           <t>44</t>
         </is>
       </c>
-      <c r="C19" s="18" t="inlineStr">
-        <is>
-          <t>《可爱的小猫》</t>
-        </is>
-      </c>
-      <c r="D19" s="18" t="inlineStr">
-        <is>
-          <t>1) 经历将“小猫乐乐”在方格纸上利用“数对”放大的探索过程，通过“填一填”“画一画”等活动，体会用“数对”的变化进行图形的放大与缩小的方法，积累数学活动经验。
-2) 在活动中体验图形的多种变化，感受在方格纸上利用“数对”进行图形的放大与缩小的趣味性，激发数学兴趣。</t>
-        </is>
-      </c>
-      <c r="E19" s="18" t="inlineStr">
+      <c r="C19" s="20" t="inlineStr">
+        <is>
+          <t>《可爱的小猫》</t>
+        </is>
+      </c>
+      <c r="D19" s="20" t="inlineStr">
+        <is>
+          <t>1) 经历将“小猫乐乐”在方格纸上利用“数对”放大的探索过程，通过“填一填”“画一画”等活动，体会用“数对”的变化进行图形的放大与缩小的方法，积累数学活动经验。
+2) 在活动中体验图形的多种变化，感受在方格纸上利用“数对”进行图形的放大与缩小的趣味性，激发数学兴趣。</t>
+        </is>
+      </c>
+      <c r="E19" s="20" t="inlineStr">
         <is>
           <t>目标1：学到=「数对前后两个点同时乘或除以一个相同的数，图形形状不变。」</t>
         </is>
       </c>
-      <c r="F19" s="18" t="inlineStr">
+      <c r="F19" s="20" t="inlineStr">
         <is>
           <t>R1 AI：你提到数对前后两个点同时乘一个相同的数图形形状不变，那么为什么这样做能保持形状不变呢？请结合具体例子说明。
     学生：「一个正方形有四个点，」
@@ -1839,45 +2465,45 @@
     学生：「扩大形成正方形」</t>
         </is>
       </c>
-      <c r="G19" s="19" t="n"/>
-      <c r="H19" s="19" t="n"/>
-      <c r="I19" s="20" t="n"/>
-      <c r="J19" s="19" t="n"/>
-      <c r="K19" s="21" t="inlineStr">
-        <is>
-          <t>T1</t>
-        </is>
-      </c>
-      <c r="L19" s="22" t="n"/>
+      <c r="G19" s="21" t="n"/>
+      <c r="H19" s="21" t="n"/>
+      <c r="I19" s="22" t="n"/>
+      <c r="J19" s="21" t="n"/>
+      <c r="K19" s="23" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="L19" s="24" t="n"/>
     </row>
     <row r="20" ht="150" customHeight="1">
-      <c r="A20" s="17" t="inlineStr">
+      <c r="A20" s="19" t="inlineStr">
         <is>
           <t>数18</t>
         </is>
       </c>
-      <c r="B20" s="18" t="inlineStr">
+      <c r="B20" s="20" t="inlineStr">
         <is>
           <t>10号</t>
         </is>
       </c>
-      <c r="C20" s="18" t="inlineStr">
-        <is>
-          <t>《可爱的小猫》</t>
-        </is>
-      </c>
-      <c r="D20" s="18" t="inlineStr">
-        <is>
-          <t>1) 经历将“小猫乐乐”在方格纸上利用“数对”放大的探索过程，通过“填一填”“画一画”等活动，体会用“数对”的变化进行图形的放大与缩小的方法，积累数学活动经验。
-2) 在活动中体验图形的多种变化，感受在方格纸上利用“数对”进行图形的放大与缩小的趣味性，激发数学兴趣。</t>
-        </is>
-      </c>
-      <c r="E20" s="18" t="inlineStr">
+      <c r="C20" s="20" t="inlineStr">
+        <is>
+          <t>《可爱的小猫》</t>
+        </is>
+      </c>
+      <c r="D20" s="20" t="inlineStr">
+        <is>
+          <t>1) 经历将“小猫乐乐”在方格纸上利用“数对”放大的探索过程，通过“填一填”“画一画”等活动，体会用“数对”的变化进行图形的放大与缩小的方法，积累数学活动经验。
+2) 在活动中体验图形的多种变化，感受在方格纸上利用“数对”进行图形的放大与缩小的趣味性，激发数学兴趣。</t>
+        </is>
+      </c>
+      <c r="E20" s="20" t="inlineStr">
         <is>
           <t>目标1：学到=「数对」</t>
         </is>
       </c>
-      <c r="F20" s="18" t="inlineStr">
+      <c r="F20" s="20" t="inlineStr">
         <is>
           <t>R1 AI：如果要将方格纸上的小猫乐乐放大到原来的2倍，它上面的点的数对会发生什么变化？请举例说明你的想法。
     学生：「数对的排列和」
@@ -1891,45 +2517,45 @@
     学生：「不行因为应是乘二而不是加二所以不可以扩大到原来的两倍」</t>
         </is>
       </c>
-      <c r="G20" s="19" t="n"/>
-      <c r="H20" s="19" t="n"/>
-      <c r="I20" s="20" t="n"/>
-      <c r="J20" s="19" t="n"/>
-      <c r="K20" s="21" t="inlineStr">
-        <is>
-          <t>T1</t>
-        </is>
-      </c>
-      <c r="L20" s="22" t="n"/>
+      <c r="G20" s="21" t="n"/>
+      <c r="H20" s="21" t="n"/>
+      <c r="I20" s="22" t="n"/>
+      <c r="J20" s="21" t="n"/>
+      <c r="K20" s="23" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="L20" s="24" t="n"/>
     </row>
     <row r="21" ht="150" customHeight="1">
-      <c r="A21" s="17" t="inlineStr">
+      <c r="A21" s="19" t="inlineStr">
         <is>
           <t>数13</t>
         </is>
       </c>
-      <c r="B21" s="18" t="inlineStr">
+      <c r="B21" s="20" t="inlineStr">
         <is>
           <t>45</t>
         </is>
       </c>
-      <c r="C21" s="18" t="inlineStr">
-        <is>
-          <t>《可爱的小猫》</t>
-        </is>
-      </c>
-      <c r="D21" s="18" t="inlineStr">
-        <is>
-          <t>1) 经历将“小猫乐乐”在方格纸上利用“数对”放大的探索过程，通过“填一填”“画一画”等活动，体会用“数对”的变化进行图形的放大与缩小的方法，积累数学活动经验。
-2) 在活动中体验图形的多种变化，感受在方格纸上利用“数对”进行图形的放大与缩小的趣味性，激发数学兴趣。</t>
-        </is>
-      </c>
-      <c r="E21" s="18" t="inlineStr">
+      <c r="C21" s="20" t="inlineStr">
+        <is>
+          <t>《可爱的小猫》</t>
+        </is>
+      </c>
+      <c r="D21" s="20" t="inlineStr">
+        <is>
+          <t>1) 经历将“小猫乐乐”在方格纸上利用“数对”放大的探索过程，通过“填一填”“画一画”等活动，体会用“数对”的变化进行图形的放大与缩小的方法，积累数学活动经验。
+2) 在活动中体验图形的多种变化，感受在方格纸上利用“数对”进行图形的放大与缩小的趣味性，激发数学兴趣。</t>
+        </is>
+      </c>
+      <c r="E21" s="20" t="inlineStr">
         <is>
           <t>目标1：学到=「数对的表示以及规律」</t>
         </is>
       </c>
-      <c r="F21" s="18" t="inlineStr">
+      <c r="F21" s="20" t="inlineStr">
         <is>
           <t>R1 AI：你说你学到了数对的规律，那么在方格纸上把一个简单图形放大时，各个顶点的数对应该如何变化？请举例说明。
     学生：「应该把x和y轴同时乘相同的数，（1，1） -》 （2，2）」
@@ -1943,45 +2569,45 @@
     学生：「点3：（2，1）， 点4：（2， 2） ，改变后：点1：（2， 1）点2：（2， 2）点3：（4， 1）， 点4（4， 2）」</t>
         </is>
       </c>
-      <c r="G21" s="19" t="n"/>
-      <c r="H21" s="19" t="n"/>
-      <c r="I21" s="20" t="n"/>
-      <c r="J21" s="19" t="n"/>
-      <c r="K21" s="21" t="inlineStr">
-        <is>
-          <t>T1</t>
-        </is>
-      </c>
-      <c r="L21" s="22" t="n"/>
+      <c r="G21" s="21" t="n"/>
+      <c r="H21" s="21" t="n"/>
+      <c r="I21" s="22" t="n"/>
+      <c r="J21" s="21" t="n"/>
+      <c r="K21" s="23" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="L21" s="24" t="n"/>
     </row>
     <row r="22" ht="150" customHeight="1">
-      <c r="A22" s="17" t="inlineStr">
+      <c r="A22" s="19" t="inlineStr">
         <is>
           <t>数20</t>
         </is>
       </c>
-      <c r="B22" s="18" t="inlineStr">
+      <c r="B22" s="20" t="inlineStr">
         <is>
           <t>22</t>
         </is>
       </c>
-      <c r="C22" s="18" t="inlineStr">
-        <is>
-          <t>《可爱的小猫》</t>
-        </is>
-      </c>
-      <c r="D22" s="18" t="inlineStr">
-        <is>
-          <t>1) 经历将“小猫乐乐”在方格纸上利用“数对”放大的探索过程，通过“填一填”“画一画”等活动，体会用“数对”的变化进行图形的放大与缩小的方法，积累数学活动经验。
-2) 在活动中体验图形的多种变化，感受在方格纸上利用“数对”进行图形的放大与缩小的趣味性，激发数学兴趣。</t>
-        </is>
-      </c>
-      <c r="E22" s="18" t="inlineStr">
+      <c r="C22" s="20" t="inlineStr">
+        <is>
+          <t>《可爱的小猫》</t>
+        </is>
+      </c>
+      <c r="D22" s="20" t="inlineStr">
+        <is>
+          <t>1) 经历将“小猫乐乐”在方格纸上利用“数对”放大的探索过程，通过“填一填”“画一画”等活动，体会用“数对”的变化进行图形的放大与缩小的方法，积累数学活动经验。
+2) 在活动中体验图形的多种变化，感受在方格纸上利用“数对”进行图形的放大与缩小的趣味性，激发数学兴趣。</t>
+        </is>
+      </c>
+      <c r="E22" s="20" t="inlineStr">
         <is>
           <t>目标1：学到=「书堆绘图」</t>
         </is>
       </c>
-      <c r="F22" s="18" t="inlineStr">
+      <c r="F22" s="20" t="inlineStr">
         <is>
           <t>R1 AI：你提到“书堆绘图”，能具体解释一下是什么意思吗？它和我们今天要学习的“用数对放大图形”可能有什么联系？
     学生：「数对将两个点连在」
@@ -1995,45 +2621,45 @@
     学生：「点数每个放大两倍」</t>
         </is>
       </c>
-      <c r="G22" s="19" t="n"/>
-      <c r="H22" s="19" t="n"/>
-      <c r="I22" s="20" t="n"/>
-      <c r="J22" s="19" t="n"/>
-      <c r="K22" s="21" t="inlineStr">
-        <is>
-          <t>T1</t>
-        </is>
-      </c>
-      <c r="L22" s="22" t="n"/>
+      <c r="G22" s="21" t="n"/>
+      <c r="H22" s="21" t="n"/>
+      <c r="I22" s="22" t="n"/>
+      <c r="J22" s="21" t="n"/>
+      <c r="K22" s="23" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="L22" s="24" t="n"/>
     </row>
     <row r="23" ht="150" customHeight="1">
-      <c r="A23" s="17" t="inlineStr">
+      <c r="A23" s="19" t="inlineStr">
         <is>
           <t>数21</t>
         </is>
       </c>
-      <c r="B23" s="18" t="inlineStr">
+      <c r="B23" s="20" t="inlineStr">
         <is>
           <t>41</t>
         </is>
       </c>
-      <c r="C23" s="18" t="inlineStr">
-        <is>
-          <t>《可爱的小猫》</t>
-        </is>
-      </c>
-      <c r="D23" s="18" t="inlineStr">
-        <is>
-          <t>1) 经历将“小猫乐乐”在方格纸上利用“数对”放大的探索过程，通过“填一填”“画一画”等活动，体会用“数对”的变化进行图形的放大与缩小的方法，积累数学活动经验。
-2) 在活动中体验图形的多种变化，感受在方格纸上利用“数对”进行图形的放大与缩小的趣味性，激发数学兴趣。</t>
-        </is>
-      </c>
-      <c r="E23" s="18" t="inlineStr">
+      <c r="C23" s="20" t="inlineStr">
+        <is>
+          <t>《可爱的小猫》</t>
+        </is>
+      </c>
+      <c r="D23" s="20" t="inlineStr">
+        <is>
+          <t>1) 经历将“小猫乐乐”在方格纸上利用“数对”放大的探索过程，通过“填一填”“画一画”等活动，体会用“数对”的变化进行图形的放大与缩小的方法，积累数学活动经验。
+2) 在活动中体验图形的多种变化，感受在方格纸上利用“数对”进行图形的放大与缩小的趣味性，激发数学兴趣。</t>
+        </is>
+      </c>
+      <c r="E23" s="20" t="inlineStr">
         <is>
           <t>目标1：学到=「知识」；疑问=「1加1为什么=2」</t>
         </is>
       </c>
-      <c r="F23" s="18" t="inlineStr">
+      <c r="F23" s="20" t="inlineStr">
         <is>
           <t>R1 AI：你说你学到了知识，那关于用数对放大图形，你具体学到了什么知识呢？
     学生：「一个图形等比例放大后」
@@ -2043,45 +2669,45 @@
     学生：「6,4」</t>
         </is>
       </c>
-      <c r="G23" s="19" t="n"/>
-      <c r="H23" s="19" t="n"/>
-      <c r="I23" s="20" t="n"/>
-      <c r="J23" s="19" t="n"/>
-      <c r="K23" s="21" t="inlineStr">
-        <is>
-          <t>T1</t>
-        </is>
-      </c>
-      <c r="L23" s="22" t="n"/>
+      <c r="G23" s="21" t="n"/>
+      <c r="H23" s="21" t="n"/>
+      <c r="I23" s="22" t="n"/>
+      <c r="J23" s="21" t="n"/>
+      <c r="K23" s="23" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="L23" s="24" t="n"/>
     </row>
     <row r="24" ht="150" customHeight="1">
-      <c r="A24" s="17" t="inlineStr">
+      <c r="A24" s="19" t="inlineStr">
         <is>
           <t>数11</t>
         </is>
       </c>
-      <c r="B24" s="18" t="inlineStr">
+      <c r="B24" s="20" t="inlineStr">
         <is>
           <t>21</t>
         </is>
       </c>
-      <c r="C24" s="18" t="inlineStr">
-        <is>
-          <t>《可爱的小猫》</t>
-        </is>
-      </c>
-      <c r="D24" s="18" t="inlineStr">
-        <is>
-          <t>1) 经历将“小猫乐乐”在方格纸上利用“数对”放大的探索过程，通过“填一填”“画一画”等活动，体会用“数对”的变化进行图形的放大与缩小的方法，积累数学活动经验。
-2) 在活动中体验图形的多种变化，感受在方格纸上利用“数对”进行图形的放大与缩小的趣味性，激发数学兴趣。</t>
-        </is>
-      </c>
-      <c r="E24" s="18" t="inlineStr">
+      <c r="C24" s="20" t="inlineStr">
+        <is>
+          <t>《可爱的小猫》</t>
+        </is>
+      </c>
+      <c r="D24" s="20" t="inlineStr">
+        <is>
+          <t>1) 经历将“小猫乐乐”在方格纸上利用“数对”放大的探索过程，通过“填一填”“画一画”等活动，体会用“数对”的变化进行图形的放大与缩小的方法，积累数学活动经验。
+2) 在活动中体验图形的多种变化，感受在方格纸上利用“数对”进行图形的放大与缩小的趣味性，激发数学兴趣。</t>
+        </is>
+      </c>
+      <c r="E24" s="20" t="inlineStr">
         <is>
           <t>目标1：学到=「图形变化的规律」</t>
         </is>
       </c>
-      <c r="F24" s="18" t="inlineStr">
+      <c r="F24" s="20" t="inlineStr">
         <is>
           <t>R1 AI：你提到学习了图形变化的规律，那么在方格纸上，将小猫图形放大时，它的数对会怎样变化？请举例解释。
     学生：「将数对的前后两个数同时」
@@ -2095,45 +2721,45 @@
     学生：「（2，3）  将4和6都乘1/2」</t>
         </is>
       </c>
-      <c r="G24" s="19" t="n"/>
-      <c r="H24" s="19" t="n"/>
-      <c r="I24" s="20" t="n"/>
-      <c r="J24" s="19" t="n"/>
-      <c r="K24" s="21" t="inlineStr">
-        <is>
-          <t>T1</t>
-        </is>
-      </c>
-      <c r="L24" s="22" t="n"/>
+      <c r="G24" s="21" t="n"/>
+      <c r="H24" s="21" t="n"/>
+      <c r="I24" s="22" t="n"/>
+      <c r="J24" s="21" t="n"/>
+      <c r="K24" s="23" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="L24" s="24" t="n"/>
     </row>
     <row r="25" ht="150" customHeight="1">
-      <c r="A25" s="17" t="inlineStr">
+      <c r="A25" s="19" t="inlineStr">
         <is>
           <t>数31</t>
         </is>
       </c>
-      <c r="B25" s="18" t="inlineStr">
+      <c r="B25" s="20" t="inlineStr">
         <is>
           <t>11</t>
         </is>
       </c>
-      <c r="C25" s="18" t="inlineStr">
-        <is>
-          <t>《可爱的小猫》</t>
-        </is>
-      </c>
-      <c r="D25" s="18" t="inlineStr">
-        <is>
-          <t>1) 经历将“小猫乐乐”在方格纸上利用“数对”放大的探索过程，通过“填一填”“画一画”等活动，体会用“数对”的变化进行图形的放大与缩小的方法，积累数学活动经验。
-2) 在活动中体验图形的多种变化，感受在方格纸上利用“数对”进行图形的放大与缩小的趣味性，激发数学兴趣。</t>
-        </is>
-      </c>
-      <c r="E25" s="18" t="inlineStr">
+      <c r="C25" s="20" t="inlineStr">
+        <is>
+          <t>《可爱的小猫》</t>
+        </is>
+      </c>
+      <c r="D25" s="20" t="inlineStr">
+        <is>
+          <t>1) 经历将“小猫乐乐”在方格纸上利用“数对”放大的探索过程，通过“填一填”“画一画”等活动，体会用“数对”的变化进行图形的放大与缩小的方法，积累数学活动经验。
+2) 在活动中体验图形的多种变化，感受在方格纸上利用“数对”进行图形的放大与缩小的趣味性，激发数学兴趣。</t>
+        </is>
+      </c>
+      <c r="E25" s="20" t="inlineStr">
         <is>
           <t>目标1：学到=「数对是如何表示的，数对有什么意义，如何找数对中的规律，如何将规律变为图像」；疑问=「数对规律对图像有什么影响」</t>
         </is>
       </c>
-      <c r="F25" s="18" t="inlineStr">
+      <c r="F25" s="20" t="inlineStr">
         <is>
           <t>R1 AI：你反思中提到想知道数对规律对图像有什么影响，那么在“小猫乐乐”的活动中，你是怎样用数对的变化把图形放大的？请结合一个点举例说明。
     学生：「我发现数对中列数增加，图像扁，行数增加图像高，都增加图像相同，增加量比值相同，那图像与原来更想」
@@ -2147,45 +2773,45 @@
     学生：「（空）」</t>
         </is>
       </c>
-      <c r="G25" s="19" t="n"/>
-      <c r="H25" s="19" t="n"/>
-      <c r="I25" s="20" t="n"/>
-      <c r="J25" s="19" t="n"/>
-      <c r="K25" s="21" t="inlineStr">
-        <is>
-          <t>T1</t>
-        </is>
-      </c>
-      <c r="L25" s="22" t="n"/>
+      <c r="G25" s="21" t="n"/>
+      <c r="H25" s="21" t="n"/>
+      <c r="I25" s="22" t="n"/>
+      <c r="J25" s="21" t="n"/>
+      <c r="K25" s="23" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="L25" s="24" t="n"/>
     </row>
     <row r="26" ht="150" customHeight="1">
-      <c r="A26" s="17" t="inlineStr">
+      <c r="A26" s="19" t="inlineStr">
         <is>
           <t>数26</t>
         </is>
       </c>
-      <c r="B26" s="18" t="inlineStr">
+      <c r="B26" s="20" t="inlineStr">
         <is>
           <t>48</t>
         </is>
       </c>
-      <c r="C26" s="18" t="inlineStr">
-        <is>
-          <t>《可爱的小猫》</t>
-        </is>
-      </c>
-      <c r="D26" s="18" t="inlineStr">
-        <is>
-          <t>1) 经历将“小猫乐乐”在方格纸上利用“数对”放大的探索过程，通过“填一填”“画一画”等活动，体会用“数对”的变化进行图形的放大与缩小的方法，积累数学活动经验。
-2) 在活动中体验图形的多种变化，感受在方格纸上利用“数对”进行图形的放大与缩小的趣味性，激发数学兴趣。</t>
-        </is>
-      </c>
-      <c r="E26" s="18" t="inlineStr">
+      <c r="C26" s="20" t="inlineStr">
+        <is>
+          <t>《可爱的小猫》</t>
+        </is>
+      </c>
+      <c r="D26" s="20" t="inlineStr">
+        <is>
+          <t>1) 经历将“小猫乐乐”在方格纸上利用“数对”放大的探索过程，通过“填一填”“画一画”等活动，体会用“数对”的变化进行图形的放大与缩小的方法，积累数学活动经验。
+2) 在活动中体验图形的多种变化，感受在方格纸上利用“数对”进行图形的放大与缩小的趣味性，激发数学兴趣。</t>
+        </is>
+      </c>
+      <c r="E26" s="20" t="inlineStr">
         <is>
           <t>目标1：学到=「数学知识  语文知识」；疑问=「怎么样考试慢分」</t>
         </is>
       </c>
-      <c r="F26" s="18" t="inlineStr">
+      <c r="F26" s="20" t="inlineStr">
         <is>
           <t>R1 AI：在方格纸上，要把小猫乐乐的图形放大，它的每个点的数对会发生怎样的变化？请举例说明。
     学生：「会直接乘一个数」
@@ -2195,45 +2821,45 @@
     学生：「横着放大前面的乘2从3变成6」</t>
         </is>
       </c>
-      <c r="G26" s="19" t="n"/>
-      <c r="H26" s="19" t="n"/>
-      <c r="I26" s="20" t="n"/>
-      <c r="J26" s="19" t="n"/>
-      <c r="K26" s="21" t="inlineStr">
-        <is>
-          <t>T1</t>
-        </is>
-      </c>
-      <c r="L26" s="22" t="n"/>
+      <c r="G26" s="21" t="n"/>
+      <c r="H26" s="21" t="n"/>
+      <c r="I26" s="22" t="n"/>
+      <c r="J26" s="21" t="n"/>
+      <c r="K26" s="23" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="L26" s="24" t="n"/>
     </row>
     <row r="27" ht="150" customHeight="1">
-      <c r="A27" s="17" t="inlineStr">
+      <c r="A27" s="19" t="inlineStr">
         <is>
           <t>数10</t>
         </is>
       </c>
-      <c r="B27" s="18" t="inlineStr">
+      <c r="B27" s="20" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="C27" s="18" t="inlineStr">
-        <is>
-          <t>《可爱的小猫》</t>
-        </is>
-      </c>
-      <c r="D27" s="18" t="inlineStr">
-        <is>
-          <t>1) 经历将“小猫乐乐”在方格纸上利用“数对”放大的探索过程，通过“填一填”“画一画”等活动，体会用“数对”的变化进行图形的放大与缩小的方法，积累数学活动经验。
-2) 在活动中体验图形的多种变化，感受在方格纸上利用“数对”进行图形的放大与缩小的趣味性，激发数学兴趣。</t>
-        </is>
-      </c>
-      <c r="E27" s="18" t="inlineStr">
+      <c r="C27" s="20" t="inlineStr">
+        <is>
+          <t>《可爱的小猫》</t>
+        </is>
+      </c>
+      <c r="D27" s="20" t="inlineStr">
+        <is>
+          <t>1) 经历将“小猫乐乐”在方格纸上利用“数对”放大的探索过程，通过“填一填”“画一画”等活动，体会用“数对”的变化进行图形的放大与缩小的方法，积累数学活动经验。
+2) 在活动中体验图形的多种变化，感受在方格纸上利用“数对”进行图形的放大与缩小的趣味性，激发数学兴趣。</t>
+        </is>
+      </c>
+      <c r="E27" s="20" t="inlineStr">
         <is>
           <t>目标1：学到=「数对变化图形也会变化」；疑问=「数对怎么变图形才不变」</t>
         </is>
       </c>
-      <c r="F27" s="18" t="inlineStr">
+      <c r="F27" s="20" t="inlineStr">
         <is>
           <t>R1 AI：在方格纸上，数对怎么变化才能使图形不变？请用例子说明你的想法。
     学生：「数对都乘」
@@ -2247,45 +2873,45 @@
     学生：「数对都乘同一个数」</t>
         </is>
       </c>
-      <c r="G27" s="19" t="n"/>
-      <c r="H27" s="19" t="n"/>
-      <c r="I27" s="20" t="n"/>
-      <c r="J27" s="19" t="n"/>
-      <c r="K27" s="21" t="inlineStr">
-        <is>
-          <t>T1</t>
-        </is>
-      </c>
-      <c r="L27" s="22" t="n"/>
+      <c r="G27" s="21" t="n"/>
+      <c r="H27" s="21" t="n"/>
+      <c r="I27" s="22" t="n"/>
+      <c r="J27" s="21" t="n"/>
+      <c r="K27" s="23" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="L27" s="24" t="n"/>
     </row>
     <row r="28" ht="150" customHeight="1">
-      <c r="A28" s="17" t="inlineStr">
+      <c r="A28" s="19" t="inlineStr">
         <is>
           <t>数22</t>
         </is>
       </c>
-      <c r="B28" s="18" t="inlineStr">
+      <c r="B28" s="20" t="inlineStr">
         <is>
           <t>38</t>
         </is>
       </c>
-      <c r="C28" s="18" t="inlineStr">
-        <is>
-          <t>《可爱的小猫》</t>
-        </is>
-      </c>
-      <c r="D28" s="18" t="inlineStr">
-        <is>
-          <t>1) 经历将“小猫乐乐”在方格纸上利用“数对”放大的探索过程，通过“填一填”“画一画”等活动，体会用“数对”的变化进行图形的放大与缩小的方法，积累数学活动经验。
-2) 在活动中体验图形的多种变化，感受在方格纸上利用“数对”进行图形的放大与缩小的趣味性，激发数学兴趣。</t>
-        </is>
-      </c>
-      <c r="E28" s="18" t="inlineStr">
+      <c r="C28" s="20" t="inlineStr">
+        <is>
+          <t>《可爱的小猫》</t>
+        </is>
+      </c>
+      <c r="D28" s="20" t="inlineStr">
+        <is>
+          <t>1) 经历将“小猫乐乐”在方格纸上利用“数对”放大的探索过程，通过“填一填”“画一画”等活动，体会用“数对”的变化进行图形的放大与缩小的方法，积累数学活动经验。
+2) 在活动中体验图形的多种变化，感受在方格纸上利用“数对”进行图形的放大与缩小的趣味性，激发数学兴趣。</t>
+        </is>
+      </c>
+      <c r="E28" s="20" t="inlineStr">
         <is>
           <t>目标1：学到=「数对的变化」</t>
         </is>
       </c>
-      <c r="F28" s="18" t="inlineStr">
+      <c r="F28" s="20" t="inlineStr">
         <is>
           <t>R1 AI：你提到“数对的变化”，那么在方格纸上，怎样改变每个点的数对才能将小猫乐乐放大？
     学生：「将数对中的数同时乘上同一个数」
@@ -2299,45 +2925,45 @@
     学生：「会，因为（2，3）2乘2，3乘3就变成了（4，9）」</t>
         </is>
       </c>
-      <c r="G28" s="19" t="n"/>
-      <c r="H28" s="19" t="n"/>
-      <c r="I28" s="20" t="n"/>
-      <c r="J28" s="19" t="n"/>
-      <c r="K28" s="21" t="inlineStr">
-        <is>
-          <t>T1</t>
-        </is>
-      </c>
-      <c r="L28" s="22" t="n"/>
+      <c r="G28" s="21" t="n"/>
+      <c r="H28" s="21" t="n"/>
+      <c r="I28" s="22" t="n"/>
+      <c r="J28" s="21" t="n"/>
+      <c r="K28" s="23" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="L28" s="24" t="n"/>
     </row>
     <row r="29" ht="150" customHeight="1">
-      <c r="A29" s="17" t="inlineStr">
+      <c r="A29" s="19" t="inlineStr">
         <is>
           <t>数28</t>
         </is>
       </c>
-      <c r="B29" s="18" t="inlineStr">
+      <c r="B29" s="20" t="inlineStr">
         <is>
           <t>18</t>
         </is>
       </c>
-      <c r="C29" s="18" t="inlineStr">
-        <is>
-          <t>《可爱的小猫》</t>
-        </is>
-      </c>
-      <c r="D29" s="18" t="inlineStr">
-        <is>
-          <t>1) 经历将“小猫乐乐”在方格纸上利用“数对”放大的探索过程，通过“填一填”“画一画”等活动，体会用“数对”的变化进行图形的放大与缩小的方法，积累数学活动经验。
-2) 在活动中体验图形的多种变化，感受在方格纸上利用“数对”进行图形的放大与缩小的趣味性，激发数学兴趣。</t>
-        </is>
-      </c>
-      <c r="E29" s="18" t="inlineStr">
+      <c r="C29" s="20" t="inlineStr">
+        <is>
+          <t>《可爱的小猫》</t>
+        </is>
+      </c>
+      <c r="D29" s="20" t="inlineStr">
+        <is>
+          <t>1) 经历将“小猫乐乐”在方格纸上利用“数对”放大的探索过程，通过“填一填”“画一画”等活动，体会用“数对”的变化进行图形的放大与缩小的方法，积累数学活动经验。
+2) 在活动中体验图形的多种变化，感受在方格纸上利用“数对”进行图形的放大与缩小的趣味性，激发数学兴趣。</t>
+        </is>
+      </c>
+      <c r="E29" s="20" t="inlineStr">
         <is>
           <t>目标1：学到=「在一个数对中，横纵数对同时乘或除以一个相同的数（0除外），图形的形状不变」</t>
         </is>
       </c>
-      <c r="F29" s="18" t="inlineStr">
+      <c r="F29" s="20" t="inlineStr">
         <is>
           <t>R1 AI：你反思中提到“横纵数对同时乘或除以一个相同的数（0除外），图形的形状不变”，为什么必须是“同时”和“相同的数”呢？如果只把横坐标乘2，纵坐标不变，图形会怎样变化？
     学生：「会比原来宽」
@@ -2351,45 +2977,45 @@
     学生：「原来这个图形的长和宽的比是1:1」</t>
         </is>
       </c>
-      <c r="G29" s="19" t="n"/>
-      <c r="H29" s="19" t="n"/>
-      <c r="I29" s="20" t="n"/>
-      <c r="J29" s="19" t="n"/>
-      <c r="K29" s="21" t="inlineStr">
-        <is>
-          <t>T1</t>
-        </is>
-      </c>
-      <c r="L29" s="22" t="n"/>
+      <c r="G29" s="21" t="n"/>
+      <c r="H29" s="21" t="n"/>
+      <c r="I29" s="22" t="n"/>
+      <c r="J29" s="21" t="n"/>
+      <c r="K29" s="23" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="L29" s="24" t="n"/>
     </row>
     <row r="30" ht="150" customHeight="1">
-      <c r="A30" s="17" t="inlineStr">
+      <c r="A30" s="19" t="inlineStr">
         <is>
           <t>数1</t>
         </is>
       </c>
-      <c r="B30" s="18" t="inlineStr">
+      <c r="B30" s="20" t="inlineStr">
         <is>
           <t>28</t>
         </is>
       </c>
-      <c r="C30" s="18" t="inlineStr">
-        <is>
-          <t>《可爱的小猫》</t>
-        </is>
-      </c>
-      <c r="D30" s="18" t="inlineStr">
-        <is>
-          <t>1) 经历将“小猫乐乐”在方格纸上利用“数对”放大的探索过程，通过“填一填”“画一画”等活动，体会用“数对”的变化进行图形的放大与缩小的方法，积累数学活动经验。
-2) 在活动中体验图形的多种变化，感受在方格纸上利用“数对”进行图形的放大与缩小的趣味性，激发数学兴趣。</t>
-        </is>
-      </c>
-      <c r="E30" s="18" t="inlineStr">
+      <c r="C30" s="20" t="inlineStr">
+        <is>
+          <t>《可爱的小猫》</t>
+        </is>
+      </c>
+      <c r="D30" s="20" t="inlineStr">
+        <is>
+          <t>1) 经历将“小猫乐乐”在方格纸上利用“数对”放大的探索过程，通过“填一填”“画一画”等活动，体会用“数对”的变化进行图形的放大与缩小的方法，积累数学活动经验。
+2) 在活动中体验图形的多种变化，感受在方格纸上利用“数对”进行图形的放大与缩小的趣味性，激发数学兴趣。</t>
+        </is>
+      </c>
+      <c r="E30" s="20" t="inlineStr">
         <is>
           <t>目标1：学到=「数对的横轴，纵轴和数对的表示方法」</t>
         </is>
       </c>
-      <c r="F30" s="18" t="inlineStr">
+      <c r="F30" s="20" t="inlineStr">
         <is>
           <t>R1 AI：你已经知道数对可以表示方格纸上的点，如果要把小猫乐乐的图形放大到原来的2倍，你认为每个点的数对应该怎样变化？请解释你的想法。
     学生：「如果是(2,8),变成（4，16）」
@@ -2397,45 +3023,45 @@
     学生：「会向上向右2格，」</t>
         </is>
       </c>
-      <c r="G30" s="19" t="n"/>
-      <c r="H30" s="19" t="n"/>
-      <c r="I30" s="20" t="n"/>
-      <c r="J30" s="19" t="n"/>
-      <c r="K30" s="21" t="inlineStr">
-        <is>
-          <t>T1</t>
-        </is>
-      </c>
-      <c r="L30" s="22" t="n"/>
+      <c r="G30" s="21" t="n"/>
+      <c r="H30" s="21" t="n"/>
+      <c r="I30" s="22" t="n"/>
+      <c r="J30" s="21" t="n"/>
+      <c r="K30" s="23" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="L30" s="24" t="n"/>
     </row>
     <row r="31" ht="150" customHeight="1">
-      <c r="A31" s="17" t="inlineStr">
+      <c r="A31" s="19" t="inlineStr">
         <is>
           <t>数17</t>
         </is>
       </c>
-      <c r="B31" s="18" t="inlineStr">
+      <c r="B31" s="20" t="inlineStr">
         <is>
           <t>31</t>
         </is>
       </c>
-      <c r="C31" s="18" t="inlineStr">
-        <is>
-          <t>《可爱的小猫》</t>
-        </is>
-      </c>
-      <c r="D31" s="18" t="inlineStr">
-        <is>
-          <t>1) 经历将“小猫乐乐”在方格纸上利用“数对”放大的探索过程，通过“填一填”“画一画”等活动，体会用“数对”的变化进行图形的放大与缩小的方法，积累数学活动经验。
-2) 在活动中体验图形的多种变化，感受在方格纸上利用“数对”进行图形的放大与缩小的趣味性，激发数学兴趣。</t>
-        </is>
-      </c>
-      <c r="E31" s="18" t="inlineStr">
+      <c r="C31" s="20" t="inlineStr">
+        <is>
+          <t>《可爱的小猫》</t>
+        </is>
+      </c>
+      <c r="D31" s="20" t="inlineStr">
+        <is>
+          <t>1) 经历将“小猫乐乐”在方格纸上利用“数对”放大的探索过程，通过“填一填”“画一画”等活动，体会用“数对”的变化进行图形的放大与缩小的方法，积累数学活动经验。
+2) 在活动中体验图形的多种变化，感受在方格纸上利用“数对”进行图形的放大与缩小的趣味性，激发数学兴趣。</t>
+        </is>
+      </c>
+      <c r="E31" s="20" t="inlineStr">
         <is>
           <t>目标1：学到=「在上课的时候学到了要按竖列再按横列的排列来写」；疑问=「有些时候找不对点要很久的时间是为什么」</t>
         </is>
       </c>
-      <c r="F31" s="18" t="inlineStr">
+      <c r="F31" s="20" t="inlineStr">
         <is>
           <t>R1 AI：你在方格纸上根据数对找点时，具体是怎样操作的？请举例说明。
     学生：「是按照竖排和横排的顺序依次往下推算」
@@ -2445,45 +3071,45 @@
     学生：「不是的要从图形的大小和数对来看」</t>
         </is>
       </c>
-      <c r="G31" s="19" t="n"/>
-      <c r="H31" s="19" t="n"/>
-      <c r="I31" s="20" t="n"/>
-      <c r="J31" s="19" t="n"/>
-      <c r="K31" s="21" t="inlineStr">
-        <is>
-          <t>T1</t>
-        </is>
-      </c>
-      <c r="L31" s="22" t="n"/>
+      <c r="G31" s="21" t="n"/>
+      <c r="H31" s="21" t="n"/>
+      <c r="I31" s="22" t="n"/>
+      <c r="J31" s="21" t="n"/>
+      <c r="K31" s="23" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="L31" s="24" t="n"/>
     </row>
     <row r="32" ht="150" customHeight="1">
-      <c r="A32" s="17" t="inlineStr">
+      <c r="A32" s="19" t="inlineStr">
         <is>
           <t>数4</t>
         </is>
       </c>
-      <c r="B32" s="18" t="inlineStr">
+      <c r="B32" s="20" t="inlineStr">
         <is>
           <t>47</t>
         </is>
       </c>
-      <c r="C32" s="18" t="inlineStr">
-        <is>
-          <t>《可爱的小猫》</t>
-        </is>
-      </c>
-      <c r="D32" s="18" t="inlineStr">
-        <is>
-          <t>1) 经历将“小猫乐乐”在方格纸上利用“数对”放大的探索过程，通过“填一填”“画一画”等活动，体会用“数对”的变化进行图形的放大与缩小的方法，积累数学活动经验。
-2) 在活动中体验图形的多种变化，感受在方格纸上利用“数对”进行图形的放大与缩小的趣味性，激发数学兴趣。</t>
-        </is>
-      </c>
-      <c r="E32" s="18" t="inlineStr">
+      <c r="C32" s="20" t="inlineStr">
+        <is>
+          <t>《可爱的小猫》</t>
+        </is>
+      </c>
+      <c r="D32" s="20" t="inlineStr">
+        <is>
+          <t>1) 经历将“小猫乐乐”在方格纸上利用“数对”放大的探索过程，通过“填一填”“画一画”等活动，体会用“数对”的变化进行图形的放大与缩小的方法，积累数学活动经验。
+2) 在活动中体验图形的多种变化，感受在方格纸上利用“数对”进行图形的放大与缩小的趣味性，激发数学兴趣。</t>
+        </is>
+      </c>
+      <c r="E32" s="20" t="inlineStr">
         <is>
           <t>目标1：学到=「如何找到数位」</t>
         </is>
       </c>
-      <c r="F32" s="18" t="inlineStr">
+      <c r="F32" s="20" t="inlineStr">
         <is>
           <t>R1 AI：在方格纸上表示小猫乐乐轮廓上的一个点，你是怎样用数对来写的？请举个例子说明。
     学生：「先找竖排在找」
@@ -2495,16 +3121,16 @@
     学生：「三表示列二表行」</t>
         </is>
       </c>
-      <c r="G32" s="19" t="n"/>
-      <c r="H32" s="19" t="n"/>
-      <c r="I32" s="20" t="n"/>
-      <c r="J32" s="19" t="n"/>
-      <c r="K32" s="21" t="inlineStr">
-        <is>
-          <t>T1</t>
-        </is>
-      </c>
-      <c r="L32" s="22" t="n"/>
+      <c r="G32" s="21" t="n"/>
+      <c r="H32" s="21" t="n"/>
+      <c r="I32" s="22" t="n"/>
+      <c r="J32" s="21" t="n"/>
+      <c r="K32" s="23" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="L32" s="24" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="3">

</xml_diff>